<commit_message>
fix: rack position layout
</commit_message>
<xml_diff>
--- a/MIP_RULE/results/model_A_piece_details.xlsx
+++ b/MIP_RULE/results/model_A_piece_details.xlsx
@@ -569,10 +569,10 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
         <v>5</v>
@@ -581,19 +581,19 @@
         <v>6.5</v>
       </c>
       <c r="J3" t="n">
-        <v>8.169999999998254</v>
+        <v>6.5</v>
       </c>
       <c r="K3" t="n">
-        <v>1.669999999998254</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>13.67999999999825</v>
+        <v>11.84</v>
       </c>
       <c r="M3" t="n">
-        <v>15.2</v>
+        <v>13.17</v>
       </c>
       <c r="N3" t="n">
-        <v>13.67999999999825</v>
+        <v>11.84</v>
       </c>
     </row>
     <row r="4">
@@ -617,7 +617,7 @@
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -629,19 +629,19 @@
         <v>11.5</v>
       </c>
       <c r="J4" t="n">
-        <v>15.2</v>
+        <v>11.5</v>
       </c>
       <c r="K4" t="n">
-        <v>3.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>21.01999999999534</v>
+        <v>17.01</v>
       </c>
       <c r="M4" t="n">
-        <v>22.85</v>
+        <v>18.53</v>
       </c>
       <c r="N4" t="n">
-        <v>21.01999999999534</v>
+        <v>17.01</v>
       </c>
     </row>
     <row r="5">
@@ -665,10 +665,10 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
         <v>15</v>
@@ -677,19 +677,19 @@
         <v>16.5</v>
       </c>
       <c r="J5" t="n">
-        <v>22.85</v>
+        <v>16.5</v>
       </c>
       <c r="K5" t="n">
-        <v>6.35</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>28.66999999999535</v>
+        <v>22.01</v>
       </c>
       <c r="M5" t="n">
-        <v>30.5</v>
+        <v>23.53</v>
       </c>
       <c r="N5" t="n">
-        <v>28.66999999999535</v>
+        <v>22.01</v>
       </c>
     </row>
     <row r="6">
@@ -713,7 +713,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -725,19 +725,19 @@
         <v>21.5</v>
       </c>
       <c r="J6" t="n">
-        <v>30.5</v>
+        <v>21.5</v>
       </c>
       <c r="K6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>36.35</v>
+        <v>27.31999999999998</v>
       </c>
       <c r="M6" t="n">
-        <v>38.18999999998079</v>
+        <v>29.15</v>
       </c>
       <c r="N6" t="n">
-        <v>36.35</v>
+        <v>27.31999999999998</v>
       </c>
     </row>
     <row r="7">
@@ -761,7 +761,7 @@
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -773,19 +773,19 @@
         <v>26.5</v>
       </c>
       <c r="J7" t="n">
-        <v>38.18999999997858</v>
+        <v>29.15</v>
       </c>
       <c r="K7" t="n">
-        <v>11.68999999997855</v>
+        <v>2.649999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>44.03999999997858</v>
+        <v>34.96999999999981</v>
       </c>
       <c r="M7" t="n">
-        <v>45.87999999997858</v>
+        <v>36.8</v>
       </c>
       <c r="N7" t="n">
-        <v>44.03999999997858</v>
+        <v>34.96999999999981</v>
       </c>
     </row>
     <row r="8">
@@ -809,10 +809,10 @@
         <v>6</v>
       </c>
       <c r="F8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" t="n">
         <v>3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>30</v>
@@ -821,19 +821,19 @@
         <v>31.5</v>
       </c>
       <c r="J8" t="n">
-        <v>45.87999999997858</v>
+        <v>31.5</v>
       </c>
       <c r="K8" t="n">
-        <v>14.37999999997855</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>52.05999999997858</v>
+        <v>37.31999999999947</v>
       </c>
       <c r="M8" t="n">
-        <v>54.23999999997858</v>
+        <v>39.15</v>
       </c>
       <c r="N8" t="n">
-        <v>52.05999999997858</v>
+        <v>37.31999999999947</v>
       </c>
     </row>
     <row r="9">
@@ -857,10 +857,10 @@
         <v>7</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
         <v>35</v>
@@ -869,19 +869,19 @@
         <v>36.5</v>
       </c>
       <c r="J9" t="n">
-        <v>54.23999999997858</v>
+        <v>39.15</v>
       </c>
       <c r="K9" t="n">
-        <v>17.73999999997858</v>
+        <v>2.649999999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>60.41999999997858</v>
+        <v>44.96999999999947</v>
       </c>
       <c r="M9" t="n">
-        <v>62.6</v>
+        <v>46.8</v>
       </c>
       <c r="N9" t="n">
-        <v>60.41999999997858</v>
+        <v>44.96999999999947</v>
       </c>
     </row>
     <row r="10">
@@ -905,7 +905,7 @@
         <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -917,19 +917,19 @@
         <v>41.5</v>
       </c>
       <c r="J10" t="n">
-        <v>62.6</v>
+        <v>41.5</v>
       </c>
       <c r="K10" t="n">
-        <v>21.1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>68.91000000000001</v>
+        <v>47.35</v>
       </c>
       <c r="M10" t="n">
-        <v>71.23</v>
+        <v>49.18999999999949</v>
       </c>
       <c r="N10" t="n">
-        <v>68.91000000000001</v>
+        <v>47.35</v>
       </c>
     </row>
     <row r="11">
@@ -953,7 +953,7 @@
         <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -965,19 +965,19 @@
         <v>46.5</v>
       </c>
       <c r="J11" t="n">
-        <v>71.23</v>
+        <v>49.18999999999949</v>
       </c>
       <c r="K11" t="n">
-        <v>24.73</v>
+        <v>2.689999999999486</v>
       </c>
       <c r="L11" t="n">
-        <v>77.54000000000001</v>
+        <v>55.03999999999949</v>
       </c>
       <c r="M11" t="n">
-        <v>79.86</v>
+        <v>56.87999999999948</v>
       </c>
       <c r="N11" t="n">
-        <v>77.54000000000001</v>
+        <v>55.03999999999949</v>
       </c>
     </row>
     <row r="12">
@@ -1001,10 +1001,10 @@
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>50</v>
@@ -1013,19 +1013,19 @@
         <v>51.5</v>
       </c>
       <c r="J12" t="n">
-        <v>79.86</v>
+        <v>51.5</v>
       </c>
       <c r="K12" t="n">
-        <v>28.36</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>86.17</v>
+        <v>57.35</v>
       </c>
       <c r="M12" t="n">
-        <v>88.48999999999999</v>
+        <v>59.18999999999949</v>
       </c>
       <c r="N12" t="n">
-        <v>86.17</v>
+        <v>57.35</v>
       </c>
     </row>
     <row r="13">
@@ -1049,10 +1049,10 @@
         <v>11</v>
       </c>
       <c r="F13" t="n">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
         <v>55</v>
@@ -1061,19 +1061,19 @@
         <v>56.5</v>
       </c>
       <c r="J13" t="n">
-        <v>88.48999999999988</v>
+        <v>59.18999999999949</v>
       </c>
       <c r="K13" t="n">
-        <v>31.98999999999988</v>
+        <v>2.689999999999486</v>
       </c>
       <c r="L13" t="n">
-        <v>94.8</v>
+        <v>65.03999999999948</v>
       </c>
       <c r="M13" t="n">
-        <v>97.11999999999988</v>
+        <v>66.87999999999948</v>
       </c>
       <c r="N13" t="n">
-        <v>94.8</v>
+        <v>65.03999999999948</v>
       </c>
     </row>
     <row r="14">
@@ -1097,7 +1097,7 @@
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1109,19 +1109,19 @@
         <v>61.5</v>
       </c>
       <c r="J14" t="n">
-        <v>97.11999999999168</v>
+        <v>61.5</v>
       </c>
       <c r="K14" t="n">
-        <v>35.61999999999168</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>103.6299999999917</v>
+        <v>67.6799999999995</v>
       </c>
       <c r="M14" t="n">
-        <v>106.15</v>
+        <v>69.8599999999995</v>
       </c>
       <c r="N14" t="n">
-        <v>103.6299999999917</v>
+        <v>67.6799999999995</v>
       </c>
     </row>
     <row r="15">
@@ -1145,7 +1145,7 @@
         <v>13</v>
       </c>
       <c r="F15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -1157,19 +1157,19 @@
         <v>66.5</v>
       </c>
       <c r="J15" t="n">
-        <v>106.15</v>
+        <v>69.8599999999995</v>
       </c>
       <c r="K15" t="n">
-        <v>39.65</v>
+        <v>3.359999999999502</v>
       </c>
       <c r="L15" t="n">
-        <v>112.6599999999917</v>
+        <v>76.03999999999951</v>
       </c>
       <c r="M15" t="n">
-        <v>115.1799999999917</v>
+        <v>78.2199999999995</v>
       </c>
       <c r="N15" t="n">
-        <v>112.6599999999917</v>
+        <v>76.03999999999951</v>
       </c>
     </row>
     <row r="16">
@@ -1193,10 +1193,10 @@
         <v>14</v>
       </c>
       <c r="F16" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16" t="n">
         <v>70</v>
@@ -1205,19 +1205,19 @@
         <v>71.5</v>
       </c>
       <c r="J16" t="n">
-        <v>115.1799999999917</v>
+        <v>71.5</v>
       </c>
       <c r="K16" t="n">
-        <v>43.67999999999168</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>121.6899999999917</v>
+        <v>77.67999999999944</v>
       </c>
       <c r="M16" t="n">
-        <v>124.2099999999917</v>
+        <v>79.85999999999945</v>
       </c>
       <c r="N16" t="n">
-        <v>121.6899999999917</v>
+        <v>77.67999999999944</v>
       </c>
     </row>
     <row r="17">
@@ -1241,31 +1241,31 @@
         <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
         <v>75</v>
       </c>
       <c r="I17" t="n">
-        <v>78.05</v>
+        <v>76.5</v>
       </c>
       <c r="J17" t="n">
-        <v>78.05</v>
+        <v>79.85999999999945</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>3.359999999999445</v>
       </c>
       <c r="L17" t="n">
-        <v>83.38999999999996</v>
+        <v>86.03999999999945</v>
       </c>
       <c r="M17" t="n">
-        <v>84.71999999999996</v>
+        <v>88.21999999999944</v>
       </c>
       <c r="N17" t="n">
-        <v>83.38999999999996</v>
+        <v>86.03999999999945</v>
       </c>
     </row>
     <row r="18">
@@ -1289,31 +1289,31 @@
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
         <v>80</v>
       </c>
       <c r="I18" t="n">
-        <v>83.05</v>
+        <v>81.5</v>
       </c>
       <c r="J18" t="n">
-        <v>84.71999999999996</v>
+        <v>81.5</v>
       </c>
       <c r="K18" t="n">
-        <v>1.669999999999945</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>90.22999999999996</v>
+        <v>87.80999999999943</v>
       </c>
       <c r="M18" t="n">
-        <v>91.75</v>
+        <v>90.12999999999943</v>
       </c>
       <c r="N18" t="n">
-        <v>90.22999999999996</v>
+        <v>87.80999999999943</v>
       </c>
     </row>
     <row r="19">
@@ -1337,31 +1337,31 @@
         <v>17</v>
       </c>
       <c r="F19" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
         <v>85</v>
       </c>
       <c r="I19" t="n">
-        <v>88.05</v>
+        <v>86.5</v>
       </c>
       <c r="J19" t="n">
-        <v>91.75</v>
+        <v>90.12999999999931</v>
       </c>
       <c r="K19" t="n">
-        <v>3.7</v>
+        <v>3.629999999999313</v>
       </c>
       <c r="L19" t="n">
-        <v>97.56999999999996</v>
+        <v>96.43999999999932</v>
       </c>
       <c r="M19" t="n">
-        <v>99.40000000000001</v>
+        <v>98.75999999999931</v>
       </c>
       <c r="N19" t="n">
-        <v>97.56999999999996</v>
+        <v>96.43999999999932</v>
       </c>
     </row>
     <row r="20">
@@ -1385,31 +1385,31 @@
         <v>18</v>
       </c>
       <c r="F20" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>90</v>
       </c>
       <c r="I20" t="n">
-        <v>93.05</v>
+        <v>91.5</v>
       </c>
       <c r="J20" t="n">
-        <v>99.40000000000001</v>
+        <v>98.75999999999931</v>
       </c>
       <c r="K20" t="n">
-        <v>6.35</v>
+        <v>7.259999999999309</v>
       </c>
       <c r="L20" t="n">
-        <v>105.22</v>
+        <v>105.0699999999993</v>
       </c>
       <c r="M20" t="n">
-        <v>107.05</v>
+        <v>107.3899999999993</v>
       </c>
       <c r="N20" t="n">
-        <v>105.22</v>
+        <v>105.0699999999993</v>
       </c>
     </row>
     <row r="21">
@@ -1433,31 +1433,31 @@
         <v>19</v>
       </c>
       <c r="F21" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
         <v>95</v>
       </c>
       <c r="I21" t="n">
-        <v>98.05</v>
+        <v>96.5</v>
       </c>
       <c r="J21" t="n">
-        <v>107.05</v>
+        <v>107.3899999999993</v>
       </c>
       <c r="K21" t="n">
-        <v>9</v>
+        <v>10.8899999999993</v>
       </c>
       <c r="L21" t="n">
-        <v>112.9</v>
+        <v>113.7</v>
       </c>
       <c r="M21" t="n">
-        <v>114.74</v>
+        <v>116.0199999999993</v>
       </c>
       <c r="N21" t="n">
-        <v>112.9</v>
+        <v>113.7</v>
       </c>
     </row>
     <row r="22">
@@ -1481,31 +1481,31 @@
         <v>20</v>
       </c>
       <c r="F22" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H22" t="n">
         <v>100</v>
       </c>
       <c r="I22" t="n">
-        <v>103.05</v>
+        <v>101.5</v>
       </c>
       <c r="J22" t="n">
-        <v>114.74</v>
+        <v>101.5</v>
       </c>
       <c r="K22" t="n">
-        <v>11.68999999999996</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>120.59</v>
+        <v>107.8099999999994</v>
       </c>
       <c r="M22" t="n">
-        <v>122.43</v>
+        <v>110.1299999999994</v>
       </c>
       <c r="N22" t="n">
-        <v>120.59</v>
+        <v>107.8099999999994</v>
       </c>
     </row>
     <row r="23">
@@ -1529,31 +1529,31 @@
         <v>21</v>
       </c>
       <c r="F23" t="n">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H23" t="n">
         <v>105</v>
       </c>
       <c r="I23" t="n">
-        <v>108.05</v>
+        <v>106.5</v>
       </c>
       <c r="J23" t="n">
-        <v>122.43</v>
+        <v>110.1299999999994</v>
       </c>
       <c r="K23" t="n">
-        <v>14.37999999999995</v>
+        <v>3.629999999999427</v>
       </c>
       <c r="L23" t="n">
-        <v>128.61</v>
+        <v>116.4399999999994</v>
       </c>
       <c r="M23" t="n">
-        <v>130.79</v>
+        <v>118.7599999999994</v>
       </c>
       <c r="N23" t="n">
-        <v>128.61</v>
+        <v>116.4399999999994</v>
       </c>
     </row>
     <row r="24">
@@ -1577,31 +1577,31 @@
         <v>22</v>
       </c>
       <c r="F24" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H24" t="n">
         <v>110</v>
       </c>
       <c r="I24" t="n">
-        <v>113.05</v>
+        <v>111.5</v>
       </c>
       <c r="J24" t="n">
-        <v>130.79</v>
+        <v>118.7599999999994</v>
       </c>
       <c r="K24" t="n">
-        <v>17.73999999999995</v>
+        <v>7.259999999999422</v>
       </c>
       <c r="L24" t="n">
-        <v>136.97</v>
+        <v>125.0699999999994</v>
       </c>
       <c r="M24" t="n">
-        <v>139.15</v>
+        <v>127.3899999999994</v>
       </c>
       <c r="N24" t="n">
-        <v>136.97</v>
+        <v>125.0699999999994</v>
       </c>
     </row>
     <row r="25">
@@ -1625,31 +1625,31 @@
         <v>23</v>
       </c>
       <c r="F25" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H25" t="n">
         <v>115</v>
       </c>
       <c r="I25" t="n">
-        <v>118.05</v>
+        <v>116.5</v>
       </c>
       <c r="J25" t="n">
-        <v>139.15</v>
+        <v>127.3899999999994</v>
       </c>
       <c r="K25" t="n">
-        <v>21.1</v>
+        <v>10.88999999999942</v>
       </c>
       <c r="L25" t="n">
-        <v>145.46</v>
+        <v>133.7</v>
       </c>
       <c r="M25" t="n">
-        <v>147.78</v>
+        <v>136.0199999999994</v>
       </c>
       <c r="N25" t="n">
-        <v>145.46</v>
+        <v>133.7</v>
       </c>
     </row>
     <row r="26">
@@ -1673,31 +1673,31 @@
         <v>24</v>
       </c>
       <c r="F26" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26" t="n">
         <v>120</v>
       </c>
       <c r="I26" t="n">
-        <v>123.05</v>
+        <v>121.5</v>
       </c>
       <c r="J26" t="n">
-        <v>147.78</v>
+        <v>121.5</v>
       </c>
       <c r="K26" t="n">
-        <v>24.72999999999996</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>154.09</v>
+        <v>128.0099999999994</v>
       </c>
       <c r="M26" t="n">
-        <v>156.41</v>
+        <v>130.5299999999994</v>
       </c>
       <c r="N26" t="n">
-        <v>154.09</v>
+        <v>128.0099999999994</v>
       </c>
     </row>
     <row r="27">
@@ -1721,31 +1721,31 @@
         <v>25</v>
       </c>
       <c r="F27" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
         <v>125</v>
       </c>
       <c r="I27" t="n">
-        <v>128.05</v>
+        <v>126.5</v>
       </c>
       <c r="J27" t="n">
-        <v>156.41</v>
+        <v>130.5299999999993</v>
       </c>
       <c r="K27" t="n">
-        <v>28.35999999999996</v>
+        <v>4.029999999999291</v>
       </c>
       <c r="L27" t="n">
-        <v>162.72</v>
+        <v>137.0399999999993</v>
       </c>
       <c r="M27" t="n">
-        <v>165.04</v>
+        <v>139.5599999999993</v>
       </c>
       <c r="N27" t="n">
-        <v>162.72</v>
+        <v>137.0399999999993</v>
       </c>
     </row>
     <row r="28">
@@ -1769,31 +1769,31 @@
         <v>26</v>
       </c>
       <c r="F28" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
         <v>130</v>
       </c>
       <c r="I28" t="n">
-        <v>133.05</v>
+        <v>131.5</v>
       </c>
       <c r="J28" t="n">
-        <v>165.04</v>
+        <v>139.5599999999993</v>
       </c>
       <c r="K28" t="n">
-        <v>31.98999999999995</v>
+        <v>8.059999999999263</v>
       </c>
       <c r="L28" t="n">
-        <v>171.35</v>
+        <v>146.0699999999993</v>
       </c>
       <c r="M28" t="n">
-        <v>173.67</v>
+        <v>148.5899999999993</v>
       </c>
       <c r="N28" t="n">
-        <v>171.35</v>
+        <v>146.0699999999993</v>
       </c>
     </row>
     <row r="29">
@@ -1817,31 +1817,31 @@
         <v>27</v>
       </c>
       <c r="F29" t="n">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H29" t="n">
         <v>135</v>
       </c>
       <c r="I29" t="n">
-        <v>138.05</v>
+        <v>136.5</v>
       </c>
       <c r="J29" t="n">
-        <v>173.67</v>
+        <v>136.5</v>
       </c>
       <c r="K29" t="n">
-        <v>35.61999999999995</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>180.1799999999999</v>
+        <v>143.0099999999995</v>
       </c>
       <c r="M29" t="n">
-        <v>182.7</v>
+        <v>145.5299999999995</v>
       </c>
       <c r="N29" t="n">
-        <v>180.1799999999999</v>
+        <v>143.0099999999995</v>
       </c>
     </row>
     <row r="30">
@@ -1865,31 +1865,31 @@
         <v>28</v>
       </c>
       <c r="F30" t="n">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
         <v>140</v>
       </c>
       <c r="I30" t="n">
-        <v>143.05</v>
+        <v>141.5</v>
       </c>
       <c r="J30" t="n">
-        <v>182.7</v>
+        <v>145.5299999999994</v>
       </c>
       <c r="K30" t="n">
-        <v>39.64999999999998</v>
+        <v>4.029999999999404</v>
       </c>
       <c r="L30" t="n">
-        <v>189.21</v>
+        <v>152.0399999999994</v>
       </c>
       <c r="M30" t="n">
-        <v>191.73</v>
+        <v>154.5599999999994</v>
       </c>
       <c r="N30" t="n">
-        <v>189.21</v>
+        <v>152.0399999999994</v>
       </c>
     </row>
     <row r="31">
@@ -1913,31 +1913,31 @@
         <v>29</v>
       </c>
       <c r="F31" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
         <v>145</v>
       </c>
       <c r="I31" t="n">
-        <v>148.05</v>
+        <v>146.5</v>
       </c>
       <c r="J31" t="n">
-        <v>191.73</v>
+        <v>154.5599999999994</v>
       </c>
       <c r="K31" t="n">
-        <v>43.67999999999995</v>
+        <v>8.059999999999377</v>
       </c>
       <c r="L31" t="n">
-        <v>198.24</v>
+        <v>161.0699999999994</v>
       </c>
       <c r="M31" t="n">
-        <v>200.76</v>
+        <v>163.5899999999994</v>
       </c>
       <c r="N31" t="n">
-        <v>207.27</v>
+        <v>170.1</v>
       </c>
     </row>
     <row r="32">
@@ -1961,31 +1961,31 @@
         <v>30</v>
       </c>
       <c r="F32" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>150</v>
       </c>
       <c r="I32" t="n">
-        <v>153.05</v>
+        <v>151.5</v>
       </c>
       <c r="J32" t="n">
-        <v>200.76</v>
+        <v>163.5899999999993</v>
       </c>
       <c r="K32" t="n">
-        <v>47.70999999999995</v>
+        <v>12.08999999999935</v>
       </c>
       <c r="L32" t="n">
-        <v>207.27</v>
+        <v>170.1</v>
       </c>
       <c r="M32" t="n">
-        <v>209.79</v>
+        <v>172.6199999999994</v>
       </c>
       <c r="N32" t="n">
-        <v>207.27</v>
+        <v>170.1</v>
       </c>
     </row>
     <row r="33">
@@ -2009,31 +2009,31 @@
         <v>31</v>
       </c>
       <c r="F33" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
         <v>155</v>
       </c>
       <c r="I33" t="n">
-        <v>159.6</v>
+        <v>158.05</v>
       </c>
       <c r="J33" t="n">
-        <v>159.6</v>
+        <v>158.05</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>164.9399999999999</v>
+        <v>163.3899999999995</v>
       </c>
       <c r="M33" t="n">
-        <v>166.2699999999999</v>
+        <v>164.7199999999995</v>
       </c>
       <c r="N33" t="n">
-        <v>164.9399999999999</v>
+        <v>163.3899999999995</v>
       </c>
     </row>
     <row r="34">
@@ -2057,31 +2057,31 @@
         <v>32</v>
       </c>
       <c r="F34" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="G34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H34" t="n">
         <v>160</v>
       </c>
       <c r="I34" t="n">
-        <v>164.6</v>
+        <v>163.05</v>
       </c>
       <c r="J34" t="n">
-        <v>166.2699999999999</v>
+        <v>163.05</v>
       </c>
       <c r="K34" t="n">
-        <v>1.669999999999874</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>171.7799999999999</v>
+        <v>168.3899999999988</v>
       </c>
       <c r="M34" t="n">
-        <v>173.3</v>
+        <v>169.7199999999988</v>
       </c>
       <c r="N34" t="n">
-        <v>178.8099999999999</v>
+        <v>175.0599999999988</v>
       </c>
     </row>
     <row r="35">
@@ -2105,31 +2105,31 @@
         <v>33</v>
       </c>
       <c r="F35" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H35" t="n">
         <v>165</v>
       </c>
       <c r="I35" t="n">
-        <v>169.6</v>
+        <v>168.05</v>
       </c>
       <c r="J35" t="n">
-        <v>173.3</v>
+        <v>169.7199999999988</v>
       </c>
       <c r="K35" t="n">
-        <v>3.7</v>
+        <v>1.669999999998822</v>
       </c>
       <c r="L35" t="n">
-        <v>178.8099999999999</v>
+        <v>175.0599999999988</v>
       </c>
       <c r="M35" t="n">
-        <v>180.3299999999999</v>
+        <v>176.3899999999988</v>
       </c>
       <c r="N35" t="n">
-        <v>178.8099999999999</v>
+        <v>175.0599999999988</v>
       </c>
     </row>
     <row r="36">
@@ -2153,31 +2153,31 @@
         <v>34</v>
       </c>
       <c r="F36" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" t="n">
         <v>170</v>
       </c>
       <c r="I36" t="n">
-        <v>174.6</v>
+        <v>173.05</v>
       </c>
       <c r="J36" t="n">
-        <v>180.3299999999999</v>
+        <v>173.05</v>
       </c>
       <c r="K36" t="n">
-        <v>5.729999999999876</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>186.15</v>
+        <v>178.5599999999988</v>
       </c>
       <c r="M36" t="n">
-        <v>187.9799999999999</v>
+        <v>180.0799999999988</v>
       </c>
       <c r="N36" t="n">
-        <v>193.8</v>
+        <v>185.5899999999988</v>
       </c>
     </row>
     <row r="37">
@@ -2201,31 +2201,31 @@
         <v>35</v>
       </c>
       <c r="F37" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" t="n">
         <v>175</v>
       </c>
       <c r="I37" t="n">
-        <v>179.6</v>
+        <v>178.05</v>
       </c>
       <c r="J37" t="n">
-        <v>187.9799999999999</v>
+        <v>180.0799999999988</v>
       </c>
       <c r="K37" t="n">
-        <v>8.379999999999882</v>
+        <v>2.029999999998779</v>
       </c>
       <c r="L37" t="n">
-        <v>193.8</v>
+        <v>185.5899999999988</v>
       </c>
       <c r="M37" t="n">
-        <v>195.6299999999999</v>
+        <v>187.1099999999988</v>
       </c>
       <c r="N37" t="n">
-        <v>193.8</v>
+        <v>185.5899999999988</v>
       </c>
     </row>
     <row r="38">
@@ -2249,31 +2249,31 @@
         <v>36</v>
       </c>
       <c r="F38" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H38" t="n">
         <v>180</v>
       </c>
       <c r="I38" t="n">
-        <v>184.6</v>
+        <v>183.05</v>
       </c>
       <c r="J38" t="n">
-        <v>195.6299999999999</v>
+        <v>183.05</v>
       </c>
       <c r="K38" t="n">
-        <v>11.02999999999989</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>201.45</v>
+        <v>188.5599999999994</v>
       </c>
       <c r="M38" t="n">
-        <v>203.2799999999999</v>
+        <v>190.0799999999994</v>
       </c>
       <c r="N38" t="n">
-        <v>201.45</v>
+        <v>188.5599999999994</v>
       </c>
     </row>
     <row r="39">
@@ -2297,31 +2297,31 @@
         <v>37</v>
       </c>
       <c r="F39" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
         <v>185</v>
       </c>
       <c r="I39" t="n">
-        <v>189.6</v>
+        <v>188.05</v>
       </c>
       <c r="J39" t="n">
-        <v>203.2799999999999</v>
+        <v>188.05</v>
       </c>
       <c r="K39" t="n">
-        <v>13.67999999999989</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>209.1299999999999</v>
+        <v>193.8699999999994</v>
       </c>
       <c r="M39" t="n">
-        <v>210.9699999999999</v>
+        <v>195.7</v>
       </c>
       <c r="N39" t="n">
-        <v>209.1299999999999</v>
+        <v>193.8699999999994</v>
       </c>
     </row>
     <row r="40">
@@ -2345,31 +2345,31 @@
         <v>38</v>
       </c>
       <c r="F40" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40" t="n">
         <v>190</v>
       </c>
       <c r="I40" t="n">
-        <v>194.6</v>
+        <v>193.05</v>
       </c>
       <c r="J40" t="n">
-        <v>210.9699999999999</v>
+        <v>195.7</v>
       </c>
       <c r="K40" t="n">
-        <v>16.36999999999989</v>
+        <v>2.649999999999977</v>
       </c>
       <c r="L40" t="n">
-        <v>216.8199999999999</v>
+        <v>201.5199999999994</v>
       </c>
       <c r="M40" t="n">
-        <v>218.6599999999999</v>
+        <v>203.35</v>
       </c>
       <c r="N40" t="n">
-        <v>216.8199999999999</v>
+        <v>201.5199999999994</v>
       </c>
     </row>
     <row r="41">
@@ -2393,31 +2393,31 @@
         <v>39</v>
       </c>
       <c r="F41" t="n">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H41" t="n">
         <v>195</v>
       </c>
       <c r="I41" t="n">
-        <v>199.6</v>
+        <v>198.05</v>
       </c>
       <c r="J41" t="n">
-        <v>218.6599999999999</v>
+        <v>198.05</v>
       </c>
       <c r="K41" t="n">
-        <v>19.05999999999989</v>
+        <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>224.8399999999999</v>
+        <v>203.8699999999994</v>
       </c>
       <c r="M41" t="n">
-        <v>227.0199999999999</v>
+        <v>205.7</v>
       </c>
       <c r="N41" t="n">
-        <v>224.8399999999999</v>
+        <v>203.8699999999994</v>
       </c>
     </row>
     <row r="42">
@@ -2441,31 +2441,31 @@
         <v>40</v>
       </c>
       <c r="F42" t="n">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H42" t="n">
         <v>200</v>
       </c>
       <c r="I42" t="n">
-        <v>204.6</v>
+        <v>203.05</v>
       </c>
       <c r="J42" t="n">
-        <v>227.0199999999999</v>
+        <v>205.7</v>
       </c>
       <c r="K42" t="n">
-        <v>22.4199999999999</v>
+        <v>2.649999999999977</v>
       </c>
       <c r="L42" t="n">
-        <v>233.2</v>
+        <v>211.5199999999994</v>
       </c>
       <c r="M42" t="n">
-        <v>235.3799999999999</v>
+        <v>213.35</v>
       </c>
       <c r="N42" t="n">
-        <v>233.2</v>
+        <v>211.5199999999994</v>
       </c>
     </row>
     <row r="43">
@@ -2489,31 +2489,31 @@
         <v>41</v>
       </c>
       <c r="F43" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="G43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" t="n">
         <v>205</v>
       </c>
       <c r="I43" t="n">
-        <v>209.6</v>
+        <v>208.05</v>
       </c>
       <c r="J43" t="n">
-        <v>235.3799999999999</v>
+        <v>208.05</v>
       </c>
       <c r="K43" t="n">
-        <v>25.77999999999992</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>241.6899999999999</v>
+        <v>213.9</v>
       </c>
       <c r="M43" t="n">
-        <v>244.0099999999999</v>
+        <v>215.7399999999993</v>
       </c>
       <c r="N43" t="n">
-        <v>241.6899999999999</v>
+        <v>213.9</v>
       </c>
     </row>
     <row r="44">
@@ -2537,31 +2537,31 @@
         <v>42</v>
       </c>
       <c r="F44" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="G44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H44" t="n">
         <v>210</v>
       </c>
       <c r="I44" t="n">
-        <v>214.6</v>
+        <v>213.05</v>
       </c>
       <c r="J44" t="n">
-        <v>244.0099999999999</v>
+        <v>215.7399999999993</v>
       </c>
       <c r="K44" t="n">
-        <v>29.40999999999991</v>
+        <v>2.689999999999259</v>
       </c>
       <c r="L44" t="n">
-        <v>250.3199999999999</v>
+        <v>221.5899999999993</v>
       </c>
       <c r="M44" t="n">
-        <v>252.6399999999999</v>
+        <v>223.4299999999993</v>
       </c>
       <c r="N44" t="n">
-        <v>250.3199999999999</v>
+        <v>221.5899999999993</v>
       </c>
     </row>
     <row r="45">
@@ -2585,31 +2585,31 @@
         <v>43</v>
       </c>
       <c r="F45" t="n">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="G45" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H45" t="n">
         <v>215</v>
       </c>
       <c r="I45" t="n">
-        <v>219.6</v>
+        <v>218.05</v>
       </c>
       <c r="J45" t="n">
-        <v>252.6399999999999</v>
+        <v>218.05</v>
       </c>
       <c r="K45" t="n">
-        <v>33.03999999999991</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>258.95</v>
+        <v>223.9</v>
       </c>
       <c r="M45" t="n">
-        <v>261.2699999999999</v>
+        <v>225.7399999999994</v>
       </c>
       <c r="N45" t="n">
-        <v>258.95</v>
+        <v>223.9</v>
       </c>
     </row>
     <row r="46">
@@ -2633,31 +2633,31 @@
         <v>44</v>
       </c>
       <c r="F46" t="n">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="G46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H46" t="n">
         <v>220</v>
       </c>
       <c r="I46" t="n">
-        <v>224.6</v>
+        <v>223.05</v>
       </c>
       <c r="J46" t="n">
-        <v>261.2699999999999</v>
+        <v>225.7399999999994</v>
       </c>
       <c r="K46" t="n">
-        <v>36.6699999999999</v>
+        <v>2.689999999999429</v>
       </c>
       <c r="L46" t="n">
-        <v>267.5799999999999</v>
+        <v>231.5899999999994</v>
       </c>
       <c r="M46" t="n">
-        <v>269.9</v>
+        <v>233.4299999999994</v>
       </c>
       <c r="N46" t="n">
-        <v>267.5799999999999</v>
+        <v>231.5899999999994</v>
       </c>
     </row>
     <row r="47">
@@ -2681,31 +2681,31 @@
         <v>45</v>
       </c>
       <c r="F47" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H47" t="n">
         <v>225</v>
       </c>
       <c r="I47" t="n">
-        <v>229.6</v>
+        <v>228.05</v>
       </c>
       <c r="J47" t="n">
-        <v>269.9</v>
+        <v>228.05</v>
       </c>
       <c r="K47" t="n">
-        <v>40.29999999999998</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>276.4099999999999</v>
+        <v>234.2299999999985</v>
       </c>
       <c r="M47" t="n">
-        <v>278.9299999999999</v>
+        <v>236.4099999999985</v>
       </c>
       <c r="N47" t="n">
-        <v>276.4099999999999</v>
+        <v>234.2299999999985</v>
       </c>
     </row>
     <row r="48">
@@ -2729,31 +2729,31 @@
         <v>46</v>
       </c>
       <c r="F48" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H48" t="n">
         <v>230</v>
       </c>
       <c r="I48" t="n">
-        <v>234.6</v>
+        <v>233.05</v>
       </c>
       <c r="J48" t="n">
-        <v>278.9299999999999</v>
+        <v>236.4099999999985</v>
       </c>
       <c r="K48" t="n">
-        <v>44.32999999999993</v>
+        <v>3.359999999998536</v>
       </c>
       <c r="L48" t="n">
-        <v>285.4399999999999</v>
+        <v>242.5899999999986</v>
       </c>
       <c r="M48" t="n">
-        <v>287.9599999999999</v>
+        <v>244.7699999999986</v>
       </c>
       <c r="N48" t="n">
-        <v>285.4399999999999</v>
+        <v>242.5899999999986</v>
       </c>
     </row>
     <row r="49">
@@ -2777,31 +2777,31 @@
         <v>47</v>
       </c>
       <c r="F49" t="n">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="G49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H49" t="n">
         <v>235</v>
       </c>
       <c r="I49" t="n">
-        <v>239.6</v>
+        <v>238.05</v>
       </c>
       <c r="J49" t="n">
-        <v>287.9599999999999</v>
+        <v>238.05</v>
       </c>
       <c r="K49" t="n">
-        <v>48.3599999999999</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>294.4699999999999</v>
+        <v>244.2299999999994</v>
       </c>
       <c r="M49" t="n">
-        <v>296.9899999999999</v>
+        <v>246.4099999999995</v>
       </c>
       <c r="N49" t="n">
-        <v>294.4699999999999</v>
+        <v>244.2299999999994</v>
       </c>
     </row>
     <row r="50">
@@ -2825,31 +2825,31 @@
         <v>48</v>
       </c>
       <c r="F50" t="n">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="G50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H50" t="n">
         <v>240</v>
       </c>
       <c r="I50" t="n">
-        <v>246.15</v>
+        <v>243.05</v>
       </c>
       <c r="J50" t="n">
-        <v>246.15</v>
+        <v>246.4099999999995</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>3.359999999999445</v>
       </c>
       <c r="L50" t="n">
-        <v>251.4899999999999</v>
+        <v>252.5899999999995</v>
       </c>
       <c r="M50" t="n">
-        <v>252.8199999999999</v>
+        <v>254.7699999999995</v>
       </c>
       <c r="N50" t="n">
-        <v>251.4899999999999</v>
+        <v>252.5899999999995</v>
       </c>
     </row>
     <row r="51">
@@ -2873,31 +2873,31 @@
         <v>49</v>
       </c>
       <c r="F51" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H51" t="n">
         <v>245</v>
       </c>
       <c r="I51" t="n">
-        <v>251.15</v>
+        <v>248.05</v>
       </c>
       <c r="J51" t="n">
-        <v>252.8199999999999</v>
+        <v>248.05</v>
       </c>
       <c r="K51" t="n">
-        <v>1.669999999999874</v>
+        <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>258.3299999999999</v>
+        <v>254.3599999999994</v>
       </c>
       <c r="M51" t="n">
-        <v>259.85</v>
+        <v>256.6799999999994</v>
       </c>
       <c r="N51" t="n">
-        <v>258.3299999999999</v>
+        <v>254.3599999999994</v>
       </c>
     </row>
     <row r="52">
@@ -2921,31 +2921,31 @@
         <v>50</v>
       </c>
       <c r="F52" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H52" t="n">
         <v>250</v>
       </c>
       <c r="I52" t="n">
-        <v>256.15</v>
+        <v>253.05</v>
       </c>
       <c r="J52" t="n">
-        <v>259.85</v>
+        <v>256.6799999999993</v>
       </c>
       <c r="K52" t="n">
-        <v>3.7</v>
+        <v>3.629999999999256</v>
       </c>
       <c r="L52" t="n">
-        <v>265.6699999999998</v>
+        <v>262.9899999999993</v>
       </c>
       <c r="M52" t="n">
-        <v>267.5</v>
+        <v>265.3099999999993</v>
       </c>
       <c r="N52" t="n">
-        <v>273.3199999999998</v>
+        <v>271.6199999999993</v>
       </c>
     </row>
     <row r="53">
@@ -2969,31 +2969,31 @@
         <v>51</v>
       </c>
       <c r="F53" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H53" t="n">
         <v>255</v>
       </c>
       <c r="I53" t="n">
-        <v>261.15</v>
+        <v>258.05</v>
       </c>
       <c r="J53" t="n">
-        <v>267.5</v>
+        <v>265.3099999999993</v>
       </c>
       <c r="K53" t="n">
-        <v>6.35</v>
+        <v>7.259999999999252</v>
       </c>
       <c r="L53" t="n">
-        <v>273.3199999999998</v>
+        <v>271.6199999999993</v>
       </c>
       <c r="M53" t="n">
-        <v>275.15</v>
+        <v>273.9399999999993</v>
       </c>
       <c r="N53" t="n">
-        <v>273.3199999999998</v>
+        <v>271.6199999999993</v>
       </c>
     </row>
     <row r="54">
@@ -3017,31 +3017,31 @@
         <v>52</v>
       </c>
       <c r="F54" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H54" t="n">
         <v>260</v>
       </c>
       <c r="I54" t="n">
-        <v>266.15</v>
+        <v>263.05</v>
       </c>
       <c r="J54" t="n">
-        <v>275.15</v>
+        <v>273.9399999999993</v>
       </c>
       <c r="K54" t="n">
-        <v>9</v>
+        <v>10.88999999999925</v>
       </c>
       <c r="L54" t="n">
-        <v>280.9699999999998</v>
+        <v>280.25</v>
       </c>
       <c r="M54" t="n">
-        <v>282.8</v>
+        <v>282.5699999999993</v>
       </c>
       <c r="N54" t="n">
-        <v>280.9699999999998</v>
+        <v>280.25</v>
       </c>
     </row>
     <row r="55">
@@ -3065,31 +3065,31 @@
         <v>53</v>
       </c>
       <c r="F55" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="G55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H55" t="n">
         <v>265</v>
       </c>
       <c r="I55" t="n">
-        <v>271.15</v>
+        <v>268.05</v>
       </c>
       <c r="J55" t="n">
-        <v>282.8</v>
+        <v>282.5699999999993</v>
       </c>
       <c r="K55" t="n">
-        <v>11.65</v>
+        <v>14.51999999999924</v>
       </c>
       <c r="L55" t="n">
-        <v>288.65</v>
+        <v>288.8799999999993</v>
       </c>
       <c r="M55" t="n">
-        <v>290.4899999999998</v>
+        <v>291.2</v>
       </c>
       <c r="N55" t="n">
-        <v>288.65</v>
+        <v>288.8799999999993</v>
       </c>
     </row>
     <row r="56">
@@ -3113,31 +3113,31 @@
         <v>54</v>
       </c>
       <c r="F56" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="G56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H56" t="n">
         <v>270</v>
       </c>
       <c r="I56" t="n">
-        <v>276.15</v>
+        <v>273.05</v>
       </c>
       <c r="J56" t="n">
-        <v>290.4899999999998</v>
+        <v>273.05</v>
       </c>
       <c r="K56" t="n">
-        <v>14.33999999999975</v>
+        <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>296.3399999999998</v>
+        <v>279.3599999999996</v>
       </c>
       <c r="M56" t="n">
-        <v>298.1799999999998</v>
+        <v>281.6799999999996</v>
       </c>
       <c r="N56" t="n">
-        <v>296.3399999999998</v>
+        <v>279.3599999999996</v>
       </c>
     </row>
     <row r="57">
@@ -3161,31 +3161,31 @@
         <v>55</v>
       </c>
       <c r="F57" t="n">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="G57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H57" t="n">
         <v>275</v>
       </c>
       <c r="I57" t="n">
-        <v>281.15</v>
+        <v>278.05</v>
       </c>
       <c r="J57" t="n">
-        <v>298.1799999999998</v>
+        <v>281.6799999999994</v>
       </c>
       <c r="K57" t="n">
-        <v>17.02999999999975</v>
+        <v>3.629999999999427</v>
       </c>
       <c r="L57" t="n">
-        <v>304.3599999999998</v>
+        <v>287.9899999999994</v>
       </c>
       <c r="M57" t="n">
-        <v>306.5399999999998</v>
+        <v>290.3099999999994</v>
       </c>
       <c r="N57" t="n">
-        <v>304.3599999999998</v>
+        <v>287.9899999999994</v>
       </c>
     </row>
     <row r="58">
@@ -3209,31 +3209,31 @@
         <v>56</v>
       </c>
       <c r="F58" t="n">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="G58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H58" t="n">
         <v>280</v>
       </c>
       <c r="I58" t="n">
-        <v>286.15</v>
+        <v>283.05</v>
       </c>
       <c r="J58" t="n">
-        <v>306.5399999999998</v>
+        <v>290.3099999999994</v>
       </c>
       <c r="K58" t="n">
-        <v>20.38999999999976</v>
+        <v>7.259999999999422</v>
       </c>
       <c r="L58" t="n">
-        <v>312.7199999999998</v>
+        <v>296.6199999999994</v>
       </c>
       <c r="M58" t="n">
-        <v>314.9</v>
+        <v>298.9399999999994</v>
       </c>
       <c r="N58" t="n">
-        <v>312.7199999999998</v>
+        <v>296.6199999999994</v>
       </c>
     </row>
     <row r="59">
@@ -3257,31 +3257,31 @@
         <v>57</v>
       </c>
       <c r="F59" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="G59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H59" t="n">
         <v>285</v>
       </c>
       <c r="I59" t="n">
-        <v>291.15</v>
+        <v>288.05</v>
       </c>
       <c r="J59" t="n">
-        <v>314.9</v>
+        <v>298.9399999999994</v>
       </c>
       <c r="K59" t="n">
-        <v>23.75</v>
+        <v>10.88999999999942</v>
       </c>
       <c r="L59" t="n">
-        <v>321.2099999999998</v>
+        <v>305.25</v>
       </c>
       <c r="M59" t="n">
-        <v>323.5299999999998</v>
+        <v>307.5699999999994</v>
       </c>
       <c r="N59" t="n">
-        <v>321.2099999999998</v>
+        <v>305.25</v>
       </c>
     </row>
     <row r="60">
@@ -3305,31 +3305,31 @@
         <v>58</v>
       </c>
       <c r="F60" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="G60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H60" t="n">
         <v>290</v>
       </c>
       <c r="I60" t="n">
-        <v>296.15</v>
+        <v>293.05</v>
       </c>
       <c r="J60" t="n">
-        <v>323.5299999999998</v>
+        <v>293.05</v>
       </c>
       <c r="K60" t="n">
-        <v>27.37999999999977</v>
+        <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>329.8399999999998</v>
+        <v>299.5599999999995</v>
       </c>
       <c r="M60" t="n">
-        <v>332.1599999999998</v>
+        <v>302.0799999999996</v>
       </c>
       <c r="N60" t="n">
-        <v>329.8399999999998</v>
+        <v>299.5599999999995</v>
       </c>
     </row>
     <row r="61">
@@ -3353,31 +3353,31 @@
         <v>59</v>
       </c>
       <c r="F61" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="G61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H61" t="n">
         <v>295</v>
       </c>
       <c r="I61" t="n">
-        <v>301.15</v>
+        <v>298.05</v>
       </c>
       <c r="J61" t="n">
-        <v>332.1599999999998</v>
+        <v>302.0799999999984</v>
       </c>
       <c r="K61" t="n">
-        <v>31.00999999999976</v>
+        <v>4.029999999998381</v>
       </c>
       <c r="L61" t="n">
-        <v>338.4699999999998</v>
+        <v>308.5899999999984</v>
       </c>
       <c r="M61" t="n">
-        <v>340.7899999999998</v>
+        <v>311.1099999999984</v>
       </c>
       <c r="N61" t="n">
-        <v>338.4699999999998</v>
+        <v>308.5899999999984</v>
       </c>
     </row>
     <row r="62">
@@ -3401,31 +3401,31 @@
         <v>60</v>
       </c>
       <c r="F62" t="n">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="G62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H62" t="n">
         <v>300</v>
       </c>
       <c r="I62" t="n">
-        <v>306.15</v>
+        <v>303.05</v>
       </c>
       <c r="J62" t="n">
-        <v>340.7899999999998</v>
+        <v>311.1099999999984</v>
       </c>
       <c r="K62" t="n">
-        <v>34.63999999999976</v>
+        <v>8.059999999998411</v>
       </c>
       <c r="L62" t="n">
-        <v>347.1</v>
+        <v>317.6199999999984</v>
       </c>
       <c r="M62" t="n">
-        <v>349.4199999999998</v>
+        <v>320.1399999999984</v>
       </c>
       <c r="N62" t="n">
-        <v>347.1</v>
+        <v>317.6199999999984</v>
       </c>
     </row>
     <row r="63">
@@ -3449,31 +3449,31 @@
         <v>61</v>
       </c>
       <c r="F63" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="G63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H63" t="n">
         <v>305</v>
       </c>
       <c r="I63" t="n">
-        <v>311.15</v>
+        <v>308.05</v>
       </c>
       <c r="J63" t="n">
-        <v>349.4199999999998</v>
+        <v>308.05</v>
       </c>
       <c r="K63" t="n">
-        <v>38.26999999999975</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>355.9299999999998</v>
+        <v>314.5599999999994</v>
       </c>
       <c r="M63" t="n">
-        <v>358.45</v>
+        <v>317.0799999999994</v>
       </c>
       <c r="N63" t="n">
-        <v>355.9299999999998</v>
+        <v>314.5599999999994</v>
       </c>
     </row>
     <row r="64">
@@ -3497,31 +3497,31 @@
         <v>62</v>
       </c>
       <c r="F64" t="n">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="G64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H64" t="n">
         <v>310</v>
       </c>
       <c r="I64" t="n">
-        <v>316.15</v>
+        <v>313.05</v>
       </c>
       <c r="J64" t="n">
-        <v>358.45</v>
+        <v>317.0799999999992</v>
       </c>
       <c r="K64" t="n">
-        <v>42.3</v>
+        <v>4.029999999999234</v>
       </c>
       <c r="L64" t="n">
-        <v>364.9599999999998</v>
+        <v>323.5899999999992</v>
       </c>
       <c r="M64" t="n">
-        <v>367.4799999999998</v>
+        <v>326.1099999999992</v>
       </c>
       <c r="N64" t="n">
-        <v>364.9599999999998</v>
+        <v>323.5899999999992</v>
       </c>
     </row>
     <row r="65">
@@ -3545,31 +3545,31 @@
         <v>63</v>
       </c>
       <c r="F65" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H65" t="n">
         <v>315</v>
       </c>
       <c r="I65" t="n">
-        <v>321.15</v>
+        <v>318.05</v>
       </c>
       <c r="J65" t="n">
-        <v>367.4799999999998</v>
+        <v>326.1099999999992</v>
       </c>
       <c r="K65" t="n">
-        <v>46.32999999999976</v>
+        <v>8.059999999999206</v>
       </c>
       <c r="L65" t="n">
-        <v>373.9899999999998</v>
+        <v>332.6199999999992</v>
       </c>
       <c r="M65" t="n">
-        <v>376.5099999999998</v>
+        <v>335.1399999999992</v>
       </c>
       <c r="N65" t="n">
-        <v>373.9899999999998</v>
+        <v>332.6199999999992</v>
       </c>
     </row>
     <row r="66">
@@ -3593,31 +3593,31 @@
         <v>64</v>
       </c>
       <c r="F66" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H66" t="n">
         <v>320</v>
       </c>
       <c r="I66" t="n">
-        <v>327.7</v>
+        <v>324.6</v>
       </c>
       <c r="J66" t="n">
-        <v>327.7</v>
+        <v>324.6</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>333.0399999999999</v>
+        <v>329.9399999999989</v>
       </c>
       <c r="M66" t="n">
-        <v>334.3699999999999</v>
+        <v>331.269999999999</v>
       </c>
       <c r="N66" t="n">
-        <v>333.0399999999999</v>
+        <v>329.9399999999989</v>
       </c>
     </row>
     <row r="67">
@@ -3641,31 +3641,31 @@
         <v>65</v>
       </c>
       <c r="F67" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H67" t="n">
         <v>325</v>
       </c>
       <c r="I67" t="n">
-        <v>332.7</v>
+        <v>329.6</v>
       </c>
       <c r="J67" t="n">
-        <v>334.3699999999999</v>
+        <v>329.6</v>
       </c>
       <c r="K67" t="n">
-        <v>1.669999999999902</v>
+        <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>339.8799999999999</v>
+        <v>334.9399999999989</v>
       </c>
       <c r="M67" t="n">
-        <v>341.4</v>
+        <v>336.269999999999</v>
       </c>
       <c r="N67" t="n">
-        <v>339.8799999999999</v>
+        <v>334.9399999999989</v>
       </c>
     </row>
     <row r="68">
@@ -3689,31 +3689,31 @@
         <v>66</v>
       </c>
       <c r="F68" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="G68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H68" t="n">
         <v>330</v>
       </c>
       <c r="I68" t="n">
-        <v>337.7</v>
+        <v>334.6</v>
       </c>
       <c r="J68" t="n">
-        <v>341.4</v>
+        <v>334.6</v>
       </c>
       <c r="K68" t="n">
-        <v>3.699999999999989</v>
+        <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>347.2199999999999</v>
+        <v>340.1099999999982</v>
       </c>
       <c r="M68" t="n">
-        <v>349.05</v>
+        <v>341.6299999999982</v>
       </c>
       <c r="N68" t="n">
-        <v>347.2199999999999</v>
+        <v>340.1099999999982</v>
       </c>
     </row>
     <row r="69">
@@ -3737,31 +3737,31 @@
         <v>67</v>
       </c>
       <c r="F69" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="G69" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H69" t="n">
         <v>335</v>
       </c>
       <c r="I69" t="n">
-        <v>342.7</v>
+        <v>339.6</v>
       </c>
       <c r="J69" t="n">
-        <v>349.05</v>
+        <v>339.6</v>
       </c>
       <c r="K69" t="n">
-        <v>6.35</v>
+        <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>354.8699999999999</v>
+        <v>345.1099999999994</v>
       </c>
       <c r="M69" t="n">
-        <v>356.7</v>
+        <v>346.6299999999994</v>
       </c>
       <c r="N69" t="n">
-        <v>354.8699999999999</v>
+        <v>345.1099999999994</v>
       </c>
     </row>
     <row r="70">
@@ -3785,31 +3785,31 @@
         <v>68</v>
       </c>
       <c r="F70" t="n">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="G70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H70" t="n">
         <v>340</v>
       </c>
       <c r="I70" t="n">
-        <v>347.7</v>
+        <v>344.6</v>
       </c>
       <c r="J70" t="n">
-        <v>356.7</v>
+        <v>344.6</v>
       </c>
       <c r="K70" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
-        <v>362.55</v>
+        <v>350.4199999999988</v>
       </c>
       <c r="M70" t="n">
-        <v>364.3899999999999</v>
+        <v>352.25</v>
       </c>
       <c r="N70" t="n">
-        <v>362.55</v>
+        <v>350.4199999999988</v>
       </c>
     </row>
     <row r="71">
@@ -3833,31 +3833,31 @@
         <v>69</v>
       </c>
       <c r="F71" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="G71" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H71" t="n">
         <v>345</v>
       </c>
       <c r="I71" t="n">
-        <v>352.7</v>
+        <v>349.6</v>
       </c>
       <c r="J71" t="n">
-        <v>364.3899999999999</v>
+        <v>352.25</v>
       </c>
       <c r="K71" t="n">
-        <v>11.68999999999983</v>
+        <v>2.649999999999977</v>
       </c>
       <c r="L71" t="n">
-        <v>370.2399999999999</v>
+        <v>358.0699999999956</v>
       </c>
       <c r="M71" t="n">
-        <v>372.0799999999999</v>
+        <v>359.9</v>
       </c>
       <c r="N71" t="n">
-        <v>370.2399999999999</v>
+        <v>358.0699999999956</v>
       </c>
     </row>
     <row r="72">
@@ -3881,31 +3881,31 @@
         <v>70</v>
       </c>
       <c r="F72" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="G72" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H72" t="n">
         <v>350</v>
       </c>
       <c r="I72" t="n">
-        <v>357.7</v>
+        <v>354.6</v>
       </c>
       <c r="J72" t="n">
-        <v>372.0799999999999</v>
+        <v>354.6</v>
       </c>
       <c r="K72" t="n">
-        <v>14.37999999999982</v>
+        <v>0</v>
       </c>
       <c r="L72" t="n">
-        <v>378.2599999999999</v>
+        <v>360.4199999999985</v>
       </c>
       <c r="M72" t="n">
-        <v>380.4399999999999</v>
+        <v>362.25</v>
       </c>
       <c r="N72" t="n">
-        <v>378.2599999999999</v>
+        <v>360.4199999999985</v>
       </c>
     </row>
     <row r="73">
@@ -3929,31 +3929,31 @@
         <v>71</v>
       </c>
       <c r="F73" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="G73" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H73" t="n">
         <v>355</v>
       </c>
       <c r="I73" t="n">
-        <v>362.7</v>
+        <v>359.6</v>
       </c>
       <c r="J73" t="n">
-        <v>380.4399999999999</v>
+        <v>362.25</v>
       </c>
       <c r="K73" t="n">
-        <v>17.73999999999984</v>
+        <v>2.649999999999977</v>
       </c>
       <c r="L73" t="n">
-        <v>386.6199999999999</v>
+        <v>368.0699999999964</v>
       </c>
       <c r="M73" t="n">
-        <v>388.8</v>
+        <v>369.9</v>
       </c>
       <c r="N73" t="n">
-        <v>386.6199999999999</v>
+        <v>368.0699999999964</v>
       </c>
     </row>
     <row r="74">
@@ -3977,31 +3977,31 @@
         <v>72</v>
       </c>
       <c r="F74" t="n">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="G74" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H74" t="n">
         <v>360</v>
       </c>
       <c r="I74" t="n">
-        <v>367.7</v>
+        <v>364.6</v>
       </c>
       <c r="J74" t="n">
-        <v>388.8</v>
+        <v>364.6</v>
       </c>
       <c r="K74" t="n">
-        <v>21.1</v>
+        <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>395.1099999999999</v>
+        <v>370.45</v>
       </c>
       <c r="M74" t="n">
-        <v>397.4299999999999</v>
+        <v>372.2899999999983</v>
       </c>
       <c r="N74" t="n">
-        <v>395.1099999999999</v>
+        <v>370.45</v>
       </c>
     </row>
     <row r="75">
@@ -4025,31 +4025,31 @@
         <v>73</v>
       </c>
       <c r="F75" t="n">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="G75" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H75" t="n">
         <v>365</v>
       </c>
       <c r="I75" t="n">
-        <v>372.7</v>
+        <v>369.6</v>
       </c>
       <c r="J75" t="n">
-        <v>397.4299999999999</v>
+        <v>372.2899999999965</v>
       </c>
       <c r="K75" t="n">
-        <v>24.72999999999985</v>
+        <v>2.689999999996473</v>
       </c>
       <c r="L75" t="n">
-        <v>403.7399999999999</v>
+        <v>378.1399999999965</v>
       </c>
       <c r="M75" t="n">
-        <v>406.0599999999999</v>
+        <v>379.9799999999965</v>
       </c>
       <c r="N75" t="n">
-        <v>403.7399999999999</v>
+        <v>378.1399999999965</v>
       </c>
     </row>
     <row r="76">
@@ -4073,31 +4073,31 @@
         <v>74</v>
       </c>
       <c r="F76" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G76" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H76" t="n">
         <v>370</v>
       </c>
       <c r="I76" t="n">
-        <v>377.7</v>
+        <v>374.6</v>
       </c>
       <c r="J76" t="n">
-        <v>406.0599999999999</v>
+        <v>374.6</v>
       </c>
       <c r="K76" t="n">
-        <v>28.35999999999984</v>
+        <v>0</v>
       </c>
       <c r="L76" t="n">
-        <v>412.3699999999999</v>
+        <v>380.45</v>
       </c>
       <c r="M76" t="n">
-        <v>414.6899999999999</v>
+        <v>382.2899999999985</v>
       </c>
       <c r="N76" t="n">
-        <v>412.3699999999999</v>
+        <v>380.45</v>
       </c>
     </row>
     <row r="77">
@@ -4121,31 +4121,31 @@
         <v>75</v>
       </c>
       <c r="F77" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="G77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H77" t="n">
         <v>375</v>
       </c>
       <c r="I77" t="n">
-        <v>382.7</v>
+        <v>379.6</v>
       </c>
       <c r="J77" t="n">
-        <v>414.6899999999999</v>
+        <v>382.2899999999952</v>
       </c>
       <c r="K77" t="n">
-        <v>31.98999999999984</v>
+        <v>2.689999999995223</v>
       </c>
       <c r="L77" t="n">
-        <v>421</v>
+        <v>388.1399999999953</v>
       </c>
       <c r="M77" t="n">
-        <v>423.3199999999999</v>
+        <v>389.9799999999952</v>
       </c>
       <c r="N77" t="n">
-        <v>421</v>
+        <v>388.1399999999953</v>
       </c>
     </row>
     <row r="78">
@@ -4169,31 +4169,31 @@
         <v>76</v>
       </c>
       <c r="F78" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="G78" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H78" t="n">
         <v>380</v>
       </c>
       <c r="I78" t="n">
-        <v>387.7</v>
+        <v>384.6</v>
       </c>
       <c r="J78" t="n">
-        <v>423.3199999999999</v>
+        <v>384.6</v>
       </c>
       <c r="K78" t="n">
-        <v>35.61999999999983</v>
+        <v>0</v>
       </c>
       <c r="L78" t="n">
-        <v>429.8299999999999</v>
+        <v>390.779999999998</v>
       </c>
       <c r="M78" t="n">
-        <v>432.35</v>
+        <v>392.959999999998</v>
       </c>
       <c r="N78" t="n">
-        <v>429.8299999999999</v>
+        <v>390.779999999998</v>
       </c>
     </row>
     <row r="79">
@@ -4217,31 +4217,31 @@
         <v>77</v>
       </c>
       <c r="F79" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H79" t="n">
         <v>385</v>
       </c>
       <c r="I79" t="n">
-        <v>392.7</v>
+        <v>389.6</v>
       </c>
       <c r="J79" t="n">
-        <v>432.35</v>
+        <v>392.9599999999962</v>
       </c>
       <c r="K79" t="n">
-        <v>39.65</v>
+        <v>3.359999999996148</v>
       </c>
       <c r="L79" t="n">
-        <v>438.8599999999999</v>
+        <v>399.1399999999962</v>
       </c>
       <c r="M79" t="n">
-        <v>441.3799999999999</v>
+        <v>401.3199999999962</v>
       </c>
       <c r="N79" t="n">
-        <v>438.8599999999999</v>
+        <v>399.1399999999962</v>
       </c>
     </row>
     <row r="80">
@@ -4265,31 +4265,31 @@
         <v>78</v>
       </c>
       <c r="F80" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H80" t="n">
         <v>390</v>
       </c>
       <c r="I80" t="n">
-        <v>397.7</v>
+        <v>394.6</v>
       </c>
       <c r="J80" t="n">
-        <v>441.3799999999999</v>
+        <v>394.6</v>
       </c>
       <c r="K80" t="n">
-        <v>43.67999999999984</v>
+        <v>0</v>
       </c>
       <c r="L80" t="n">
-        <v>447.8899999999999</v>
+        <v>400.7799999999984</v>
       </c>
       <c r="M80" t="n">
-        <v>450.4099999999999</v>
+        <v>402.9599999999984</v>
       </c>
       <c r="N80" t="n">
-        <v>447.8899999999999</v>
+        <v>400.7799999999984</v>
       </c>
     </row>
     <row r="81">
@@ -4313,7 +4313,7 @@
         <v>79</v>
       </c>
       <c r="F81" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="G81" t="n">
         <v>5</v>
@@ -4322,22 +4322,22 @@
         <v>395</v>
       </c>
       <c r="I81" t="n">
-        <v>404.25</v>
+        <v>399.6</v>
       </c>
       <c r="J81" t="n">
-        <v>404.25</v>
+        <v>402.9599999999949</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>3.359999999994898</v>
       </c>
       <c r="L81" t="n">
-        <v>409.5899999999997</v>
+        <v>409.1399999999949</v>
       </c>
       <c r="M81" t="n">
-        <v>410.9199999999998</v>
+        <v>411.3199999999949</v>
       </c>
       <c r="N81" t="n">
-        <v>409.5899999999997</v>
+        <v>409.1399999999949</v>
       </c>
     </row>
     <row r="82">
@@ -4361,31 +4361,31 @@
         <v>80</v>
       </c>
       <c r="F82" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="G82" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H82" t="n">
         <v>400</v>
       </c>
       <c r="I82" t="n">
-        <v>409.25</v>
+        <v>404.6</v>
       </c>
       <c r="J82" t="n">
-        <v>410.9199999999998</v>
+        <v>404.6</v>
       </c>
       <c r="K82" t="n">
-        <v>1.669999999999789</v>
+        <v>0</v>
       </c>
       <c r="L82" t="n">
-        <v>416.4299999999998</v>
+        <v>410.909999999998</v>
       </c>
       <c r="M82" t="n">
-        <v>417.95</v>
+        <v>413.229999999998</v>
       </c>
       <c r="N82" t="n">
-        <v>416.4299999999998</v>
+        <v>410.909999999998</v>
       </c>
     </row>
     <row r="83">
@@ -4409,31 +4409,31 @@
         <v>81</v>
       </c>
       <c r="F83" t="n">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="G83" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H83" t="n">
         <v>405</v>
       </c>
       <c r="I83" t="n">
-        <v>414.25</v>
+        <v>409.6</v>
       </c>
       <c r="J83" t="n">
-        <v>417.95</v>
+        <v>413.229999999996</v>
       </c>
       <c r="K83" t="n">
-        <v>3.699999999999989</v>
+        <v>3.629999999996016</v>
       </c>
       <c r="L83" t="n">
-        <v>423.7699999999998</v>
+        <v>419.539999999996</v>
       </c>
       <c r="M83" t="n">
-        <v>425.6</v>
+        <v>421.859999999996</v>
       </c>
       <c r="N83" t="n">
-        <v>423.7699999999998</v>
+        <v>419.539999999996</v>
       </c>
     </row>
     <row r="84">
@@ -4457,31 +4457,31 @@
         <v>82</v>
       </c>
       <c r="F84" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="G84" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H84" t="n">
         <v>410</v>
       </c>
       <c r="I84" t="n">
-        <v>419.25</v>
+        <v>414.6</v>
       </c>
       <c r="J84" t="n">
-        <v>425.6</v>
+        <v>421.8599999999959</v>
       </c>
       <c r="K84" t="n">
-        <v>6.35</v>
+        <v>7.259999999995898</v>
       </c>
       <c r="L84" t="n">
-        <v>431.4199999999997</v>
+        <v>428.1699999999959</v>
       </c>
       <c r="M84" t="n">
-        <v>433.25</v>
+        <v>430.4899999999959</v>
       </c>
       <c r="N84" t="n">
-        <v>431.4199999999997</v>
+        <v>428.1699999999959</v>
       </c>
     </row>
     <row r="85">
@@ -4505,31 +4505,31 @@
         <v>83</v>
       </c>
       <c r="F85" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="G85" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H85" t="n">
         <v>415</v>
       </c>
       <c r="I85" t="n">
-        <v>424.25</v>
+        <v>419.6</v>
       </c>
       <c r="J85" t="n">
-        <v>433.25</v>
+        <v>430.4899999999959</v>
       </c>
       <c r="K85" t="n">
-        <v>9</v>
+        <v>10.88999999999589</v>
       </c>
       <c r="L85" t="n">
-        <v>439.1</v>
+        <v>436.8</v>
       </c>
       <c r="M85" t="n">
-        <v>440.9399999999997</v>
+        <v>439.1199999999959</v>
       </c>
       <c r="N85" t="n">
-        <v>439.1</v>
+        <v>436.8</v>
       </c>
     </row>
     <row r="86">
@@ -4553,7 +4553,7 @@
         <v>84</v>
       </c>
       <c r="F86" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G86" t="n">
         <v>5</v>
@@ -4562,22 +4562,22 @@
         <v>420</v>
       </c>
       <c r="I86" t="n">
-        <v>429.25</v>
+        <v>424.6</v>
       </c>
       <c r="J86" t="n">
-        <v>440.9399999999997</v>
+        <v>424.6</v>
       </c>
       <c r="K86" t="n">
-        <v>11.68999999999971</v>
+        <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>446.7899999999997</v>
+        <v>430.9099999999978</v>
       </c>
       <c r="M86" t="n">
-        <v>448.6299999999997</v>
+        <v>433.2299999999977</v>
       </c>
       <c r="N86" t="n">
-        <v>446.7899999999997</v>
+        <v>430.9099999999978</v>
       </c>
     </row>
     <row r="87">
@@ -4601,7 +4601,7 @@
         <v>85</v>
       </c>
       <c r="F87" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G87" t="n">
         <v>5</v>
@@ -4610,22 +4610,22 @@
         <v>425</v>
       </c>
       <c r="I87" t="n">
-        <v>434.25</v>
+        <v>429.6</v>
       </c>
       <c r="J87" t="n">
-        <v>448.6299999999997</v>
+        <v>433.2299999999939</v>
       </c>
       <c r="K87" t="n">
-        <v>14.37999999999971</v>
+        <v>3.629999999993913</v>
       </c>
       <c r="L87" t="n">
-        <v>454.8099999999997</v>
+        <v>439.5399999999939</v>
       </c>
       <c r="M87" t="n">
-        <v>456.9899999999997</v>
+        <v>441.8599999999939</v>
       </c>
       <c r="N87" t="n">
-        <v>454.8099999999997</v>
+        <v>439.5399999999939</v>
       </c>
     </row>
     <row r="88">
@@ -4649,7 +4649,7 @@
         <v>86</v>
       </c>
       <c r="F88" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G88" t="n">
         <v>5</v>
@@ -4658,22 +4658,22 @@
         <v>430</v>
       </c>
       <c r="I88" t="n">
-        <v>439.25</v>
+        <v>434.6</v>
       </c>
       <c r="J88" t="n">
-        <v>456.9899999999997</v>
+        <v>441.8599999999911</v>
       </c>
       <c r="K88" t="n">
-        <v>17.73999999999972</v>
+        <v>7.259999999991123</v>
       </c>
       <c r="L88" t="n">
-        <v>463.1699999999997</v>
+        <v>448.1699999999911</v>
       </c>
       <c r="M88" t="n">
-        <v>465.35</v>
+        <v>450.4899999999911</v>
       </c>
       <c r="N88" t="n">
-        <v>463.1699999999997</v>
+        <v>448.1699999999911</v>
       </c>
     </row>
     <row r="89">
@@ -4697,7 +4697,7 @@
         <v>87</v>
       </c>
       <c r="F89" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G89" t="n">
         <v>5</v>
@@ -4706,22 +4706,22 @@
         <v>435</v>
       </c>
       <c r="I89" t="n">
-        <v>444.25</v>
+        <v>439.6</v>
       </c>
       <c r="J89" t="n">
-        <v>465.35</v>
+        <v>450.4899999999911</v>
       </c>
       <c r="K89" t="n">
-        <v>21.1</v>
+        <v>10.88999999999112</v>
       </c>
       <c r="L89" t="n">
-        <v>471.6599999999997</v>
+        <v>456.8</v>
       </c>
       <c r="M89" t="n">
-        <v>473.9799999999997</v>
+        <v>459.1199999999911</v>
       </c>
       <c r="N89" t="n">
-        <v>471.6599999999997</v>
+        <v>456.8</v>
       </c>
     </row>
     <row r="90">
@@ -4745,7 +4745,7 @@
         <v>88</v>
       </c>
       <c r="F90" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G90" t="n">
         <v>5</v>
@@ -4754,22 +4754,22 @@
         <v>440</v>
       </c>
       <c r="I90" t="n">
-        <v>449.25</v>
+        <v>444.6</v>
       </c>
       <c r="J90" t="n">
-        <v>473.9799999999997</v>
+        <v>459.1199999999911</v>
       </c>
       <c r="K90" t="n">
-        <v>24.72999999999973</v>
+        <v>14.51999999999111</v>
       </c>
       <c r="L90" t="n">
-        <v>480.2899999999997</v>
+        <v>465.6299999999911</v>
       </c>
       <c r="M90" t="n">
-        <v>482.6099999999997</v>
+        <v>468.15</v>
       </c>
       <c r="N90" t="n">
-        <v>559.1599999999996</v>
+        <v>519.8099999999906</v>
       </c>
     </row>
     <row r="91">
@@ -4793,7 +4793,7 @@
         <v>89</v>
       </c>
       <c r="F91" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G91" t="n">
         <v>5</v>
@@ -4802,22 +4802,22 @@
         <v>445</v>
       </c>
       <c r="I91" t="n">
-        <v>454.25</v>
+        <v>449.6</v>
       </c>
       <c r="J91" t="n">
-        <v>482.6099999999997</v>
+        <v>468.15</v>
       </c>
       <c r="K91" t="n">
-        <v>28.35999999999973</v>
+        <v>18.54999999999995</v>
       </c>
       <c r="L91" t="n">
-        <v>488.9199999999997</v>
+        <v>474.6599999999911</v>
       </c>
       <c r="M91" t="n">
-        <v>491.2399999999997</v>
+        <v>477.1799999999911</v>
       </c>
       <c r="N91" t="n">
-        <v>567.7899999999997</v>
+        <v>528.8399999999906</v>
       </c>
     </row>
     <row r="92">
@@ -4841,7 +4841,7 @@
         <v>90</v>
       </c>
       <c r="F92" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G92" t="n">
         <v>5</v>
@@ -4850,22 +4850,22 @@
         <v>450</v>
       </c>
       <c r="I92" t="n">
-        <v>459.25</v>
+        <v>454.6</v>
       </c>
       <c r="J92" t="n">
-        <v>491.2399999999997</v>
+        <v>477.1799999999911</v>
       </c>
       <c r="K92" t="n">
-        <v>31.98999999999972</v>
+        <v>22.57999999999106</v>
       </c>
       <c r="L92" t="n">
-        <v>497.55</v>
+        <v>483.6899999999911</v>
       </c>
       <c r="M92" t="n">
-        <v>499.8699999999997</v>
+        <v>486.2099999999911</v>
       </c>
       <c r="N92" t="n">
-        <v>603.1099999999997</v>
+        <v>546.9</v>
       </c>
     </row>
     <row r="93">
@@ -4889,31 +4889,31 @@
         <v>91</v>
       </c>
       <c r="F93" t="n">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="G93" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H93" t="n">
         <v>455</v>
       </c>
       <c r="I93" t="n">
-        <v>464.25</v>
+        <v>459.6</v>
       </c>
       <c r="J93" t="n">
-        <v>499.8699999999997</v>
+        <v>459.6</v>
       </c>
       <c r="K93" t="n">
-        <v>35.61999999999972</v>
+        <v>0</v>
       </c>
       <c r="L93" t="n">
-        <v>506.3799999999997</v>
+        <v>466.1099999999994</v>
       </c>
       <c r="M93" t="n">
-        <v>508.9</v>
+        <v>468.6299999999994</v>
       </c>
       <c r="N93" t="n">
-        <v>506.3799999999997</v>
+        <v>466.1099999999994</v>
       </c>
     </row>
     <row r="94">
@@ -4937,31 +4937,31 @@
         <v>92</v>
       </c>
       <c r="F94" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="G94" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H94" t="n">
         <v>460</v>
       </c>
       <c r="I94" t="n">
-        <v>469.25</v>
+        <v>464.6</v>
       </c>
       <c r="J94" t="n">
-        <v>508.9</v>
+        <v>468.629999999995</v>
       </c>
       <c r="K94" t="n">
-        <v>39.64999999999998</v>
+        <v>4.02999999999497</v>
       </c>
       <c r="L94" t="n">
-        <v>515.4099999999997</v>
+        <v>475.139999999995</v>
       </c>
       <c r="M94" t="n">
-        <v>517.9299999999997</v>
+        <v>477.659999999995</v>
       </c>
       <c r="N94" t="n">
-        <v>576.6199999999997</v>
+        <v>506.1099999999994</v>
       </c>
     </row>
     <row r="95">
@@ -4985,31 +4985,31 @@
         <v>93</v>
       </c>
       <c r="F95" t="n">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="G95" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H95" t="n">
         <v>465</v>
       </c>
       <c r="I95" t="n">
-        <v>474.25</v>
+        <v>469.6</v>
       </c>
       <c r="J95" t="n">
-        <v>517.9299999999997</v>
+        <v>477.659999999995</v>
       </c>
       <c r="K95" t="n">
-        <v>43.67999999999972</v>
+        <v>8.059999999994943</v>
       </c>
       <c r="L95" t="n">
-        <v>524.4399999999997</v>
+        <v>484.169999999995</v>
       </c>
       <c r="M95" t="n">
-        <v>526.9599999999997</v>
+        <v>486.6899999999949</v>
       </c>
       <c r="N95" t="n">
-        <v>585.65</v>
+        <v>515.1399999999983</v>
       </c>
     </row>
     <row r="96">
@@ -5033,7 +5033,7 @@
         <v>94</v>
       </c>
       <c r="F96" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G96" t="n">
         <v>5</v>
@@ -5042,22 +5042,22 @@
         <v>470</v>
       </c>
       <c r="I96" t="n">
-        <v>479.25</v>
+        <v>474.6</v>
       </c>
       <c r="J96" t="n">
-        <v>526.9599999999997</v>
+        <v>486.2099999999911</v>
       </c>
       <c r="K96" t="n">
-        <v>47.7099999999997</v>
+        <v>11.60999999999103</v>
       </c>
       <c r="L96" t="n">
-        <v>533.2699999999996</v>
+        <v>492.719999999991</v>
       </c>
       <c r="M96" t="n">
-        <v>535.5899999999997</v>
+        <v>495.239999999991</v>
       </c>
       <c r="N96" t="n">
-        <v>559.1599999999996</v>
+        <v>519.8099999999906</v>
       </c>
     </row>
     <row r="97">
@@ -5081,7 +5081,7 @@
         <v>95</v>
       </c>
       <c r="F97" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G97" t="n">
         <v>5</v>
@@ -5090,22 +5090,22 @@
         <v>475</v>
       </c>
       <c r="I97" t="n">
-        <v>484.25</v>
+        <v>479.6</v>
       </c>
       <c r="J97" t="n">
-        <v>535.5899999999997</v>
+        <v>495.239999999991</v>
       </c>
       <c r="K97" t="n">
-        <v>51.33999999999969</v>
+        <v>15.63999999999101</v>
       </c>
       <c r="L97" t="n">
-        <v>541.9</v>
+        <v>501.75</v>
       </c>
       <c r="M97" t="n">
-        <v>544.2199999999997</v>
+        <v>504.269999999991</v>
       </c>
       <c r="N97" t="n">
-        <v>567.7899999999997</v>
+        <v>528.8399999999906</v>
       </c>
     </row>
     <row r="98">
@@ -5129,7 +5129,7 @@
         <v>96</v>
       </c>
       <c r="F98" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G98" t="n">
         <v>5</v>
@@ -5138,22 +5138,22 @@
         <v>480</v>
       </c>
       <c r="I98" t="n">
-        <v>489.25</v>
+        <v>484.6</v>
       </c>
       <c r="J98" t="n">
-        <v>544.2199999999997</v>
+        <v>504.269999999991</v>
       </c>
       <c r="K98" t="n">
-        <v>54.96999999999969</v>
+        <v>19.66999999999098</v>
       </c>
       <c r="L98" t="n">
-        <v>550.5299999999996</v>
+        <v>510.779999999991</v>
       </c>
       <c r="M98" t="n">
-        <v>552.85</v>
+        <v>513.3</v>
       </c>
       <c r="N98" t="n">
-        <v>559.1599999999996</v>
+        <v>519.8099999999906</v>
       </c>
     </row>
     <row r="99">
@@ -5177,7 +5177,7 @@
         <v>97</v>
       </c>
       <c r="F99" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G99" t="n">
         <v>5</v>
@@ -5186,22 +5186,22 @@
         <v>485</v>
       </c>
       <c r="I99" t="n">
-        <v>494.25</v>
+        <v>489.6</v>
       </c>
       <c r="J99" t="n">
-        <v>552.85</v>
+        <v>513.3</v>
       </c>
       <c r="K99" t="n">
-        <v>58.6</v>
+        <v>23.69999999999993</v>
       </c>
       <c r="L99" t="n">
-        <v>559.1599999999996</v>
+        <v>519.809999999991</v>
       </c>
       <c r="M99" t="n">
-        <v>561.4799999999997</v>
+        <v>522.3299999999909</v>
       </c>
       <c r="N99" t="n">
-        <v>559.1599999999996</v>
+        <v>519.8099999999906</v>
       </c>
     </row>
     <row r="100">
@@ -5225,7 +5225,7 @@
         <v>98</v>
       </c>
       <c r="F100" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G100" t="n">
         <v>5</v>
@@ -5234,22 +5234,22 @@
         <v>490</v>
       </c>
       <c r="I100" t="n">
-        <v>499.25</v>
+        <v>494.6</v>
       </c>
       <c r="J100" t="n">
-        <v>561.4799999999997</v>
+        <v>522.3299999999909</v>
       </c>
       <c r="K100" t="n">
-        <v>62.22999999999968</v>
+        <v>27.72999999999092</v>
       </c>
       <c r="L100" t="n">
-        <v>567.7899999999997</v>
+        <v>528.8399999999909</v>
       </c>
       <c r="M100" t="n">
-        <v>570.1099999999997</v>
+        <v>531.3599999999909</v>
       </c>
       <c r="N100" t="n">
-        <v>567.7899999999997</v>
+        <v>528.8399999999906</v>
       </c>
     </row>
     <row r="101">
@@ -5273,31 +5273,31 @@
         <v>99</v>
       </c>
       <c r="F101" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="G101" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H101" t="n">
         <v>495</v>
       </c>
       <c r="I101" t="n">
-        <v>504.25</v>
+        <v>499.6</v>
       </c>
       <c r="J101" t="n">
-        <v>570.1099999999997</v>
+        <v>499.6</v>
       </c>
       <c r="K101" t="n">
-        <v>65.85999999999967</v>
+        <v>0</v>
       </c>
       <c r="L101" t="n">
-        <v>576.6199999999997</v>
+        <v>506.1099999999994</v>
       </c>
       <c r="M101" t="n">
-        <v>579.1399999999996</v>
+        <v>508.6299999999994</v>
       </c>
       <c r="N101" t="n">
-        <v>576.6199999999997</v>
+        <v>506.1099999999994</v>
       </c>
     </row>
     <row r="102">
@@ -5321,31 +5321,31 @@
         <v>100</v>
       </c>
       <c r="F102" t="n">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="G102" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H102" t="n">
         <v>500</v>
       </c>
       <c r="I102" t="n">
-        <v>509.25</v>
+        <v>504.6</v>
       </c>
       <c r="J102" t="n">
-        <v>579.1399999999996</v>
+        <v>508.6299999999983</v>
       </c>
       <c r="K102" t="n">
-        <v>69.88999999999965</v>
+        <v>4.029999999998267</v>
       </c>
       <c r="L102" t="n">
-        <v>585.65</v>
+        <v>515.1399999999983</v>
       </c>
       <c r="M102" t="n">
-        <v>588.1699999999996</v>
+        <v>517.6599999999983</v>
       </c>
       <c r="N102" t="n">
-        <v>585.65</v>
+        <v>515.1399999999983</v>
       </c>
     </row>
     <row r="103">
@@ -5369,7 +5369,7 @@
         <v>101</v>
       </c>
       <c r="F103" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G103" t="n">
         <v>5</v>
@@ -5378,22 +5378,22 @@
         <v>505</v>
       </c>
       <c r="I103" t="n">
-        <v>514.25</v>
+        <v>509.6</v>
       </c>
       <c r="J103" t="n">
-        <v>588.1699999999996</v>
+        <v>531.3599999999909</v>
       </c>
       <c r="K103" t="n">
-        <v>73.91999999999962</v>
+        <v>21.7599999999909</v>
       </c>
       <c r="L103" t="n">
-        <v>594.4799999999997</v>
+        <v>537.8699999999909</v>
       </c>
       <c r="M103" t="n">
-        <v>596.8</v>
+        <v>540.3899999999909</v>
       </c>
       <c r="N103" t="n">
-        <v>603.1099999999997</v>
+        <v>546.9</v>
       </c>
     </row>
     <row r="104">
@@ -5417,7 +5417,7 @@
         <v>101</v>
       </c>
       <c r="F104" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G104" t="n">
         <v>5</v>
@@ -5426,22 +5426,22 @@
         <v>510</v>
       </c>
       <c r="I104" t="n">
-        <v>519.25</v>
+        <v>514.6</v>
       </c>
       <c r="J104" t="n">
-        <v>596.8</v>
+        <v>540.3899999999909</v>
       </c>
       <c r="K104" t="n">
-        <v>77.54999999999995</v>
+        <v>25.78999999999087</v>
       </c>
       <c r="L104" t="n">
-        <v>603.1099999999997</v>
+        <v>546.9</v>
       </c>
       <c r="M104" t="n">
-        <v>605.4299999999996</v>
+        <v>549.4199999999909</v>
       </c>
       <c r="N104" t="n">
-        <v>603.1099999999997</v>
+        <v>546.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: objective C_k & delete amr waiting time
</commit_message>
<xml_diff>
--- a/MIP_RULE/results/model_A_piece_details.xlsx
+++ b/MIP_RULE/results/model_A_piece_details.xlsx
@@ -713,7 +713,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -731,13 +731,13 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>27.31999999999998</v>
+        <v>27.32</v>
       </c>
       <c r="M6" t="n">
         <v>29.15</v>
       </c>
       <c r="N6" t="n">
-        <v>27.31999999999998</v>
+        <v>27.32</v>
       </c>
     </row>
     <row r="7">
@@ -761,7 +761,7 @@
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -776,16 +776,16 @@
         <v>29.15</v>
       </c>
       <c r="K7" t="n">
-        <v>2.649999999999999</v>
+        <v>2.65</v>
       </c>
       <c r="L7" t="n">
-        <v>34.96999999999981</v>
+        <v>34.97000000000002</v>
       </c>
       <c r="M7" t="n">
         <v>36.8</v>
       </c>
       <c r="N7" t="n">
-        <v>34.96999999999981</v>
+        <v>34.97000000000002</v>
       </c>
     </row>
     <row r="8">
@@ -809,7 +809,7 @@
         <v>6</v>
       </c>
       <c r="F8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G8" t="n">
         <v>3</v>
@@ -827,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>37.31999999999947</v>
+        <v>37.31999999999992</v>
       </c>
       <c r="M8" t="n">
         <v>39.15</v>
       </c>
       <c r="N8" t="n">
-        <v>37.31999999999947</v>
+        <v>37.31999999999992</v>
       </c>
     </row>
     <row r="9">
@@ -857,7 +857,7 @@
         <v>7</v>
       </c>
       <c r="F9" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
         <v>3</v>
@@ -872,16 +872,16 @@
         <v>39.15</v>
       </c>
       <c r="K9" t="n">
-        <v>2.649999999999999</v>
+        <v>2.65</v>
       </c>
       <c r="L9" t="n">
-        <v>44.96999999999947</v>
+        <v>44.9699999999999</v>
       </c>
       <c r="M9" t="n">
         <v>46.8</v>
       </c>
       <c r="N9" t="n">
-        <v>44.96999999999947</v>
+        <v>44.9699999999999</v>
       </c>
     </row>
     <row r="10">
@@ -926,7 +926,7 @@
         <v>47.35</v>
       </c>
       <c r="M10" t="n">
-        <v>49.18999999999949</v>
+        <v>49.18999999999982</v>
       </c>
       <c r="N10" t="n">
         <v>47.35</v>
@@ -965,19 +965,19 @@
         <v>46.5</v>
       </c>
       <c r="J11" t="n">
-        <v>49.18999999999949</v>
+        <v>49.18999999999982</v>
       </c>
       <c r="K11" t="n">
-        <v>2.689999999999486</v>
+        <v>2.68999999999982</v>
       </c>
       <c r="L11" t="n">
-        <v>55.03999999999949</v>
+        <v>55.03999999999982</v>
       </c>
       <c r="M11" t="n">
-        <v>56.87999999999948</v>
+        <v>56.87999999999982</v>
       </c>
       <c r="N11" t="n">
-        <v>55.03999999999949</v>
+        <v>55.03999999999982</v>
       </c>
     </row>
     <row r="12">
@@ -1022,7 +1022,7 @@
         <v>57.35</v>
       </c>
       <c r="M12" t="n">
-        <v>59.18999999999949</v>
+        <v>59.18999999999966</v>
       </c>
       <c r="N12" t="n">
         <v>57.35</v>
@@ -1061,19 +1061,19 @@
         <v>56.5</v>
       </c>
       <c r="J13" t="n">
-        <v>59.18999999999949</v>
+        <v>59.18999999999966</v>
       </c>
       <c r="K13" t="n">
-        <v>2.689999999999486</v>
+        <v>2.689999999999657</v>
       </c>
       <c r="L13" t="n">
-        <v>65.03999999999948</v>
+        <v>65.03999999999965</v>
       </c>
       <c r="M13" t="n">
-        <v>66.87999999999948</v>
+        <v>66.87999999999965</v>
       </c>
       <c r="N13" t="n">
-        <v>65.03999999999948</v>
+        <v>65.03999999999965</v>
       </c>
     </row>
     <row r="14">
@@ -1115,13 +1115,13 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>67.6799999999995</v>
+        <v>67.67999999999998</v>
       </c>
       <c r="M14" t="n">
-        <v>69.8599999999995</v>
+        <v>69.85999999999997</v>
       </c>
       <c r="N14" t="n">
-        <v>67.6799999999995</v>
+        <v>67.67999999999998</v>
       </c>
     </row>
     <row r="15">
@@ -1157,19 +1157,19 @@
         <v>66.5</v>
       </c>
       <c r="J15" t="n">
-        <v>69.8599999999995</v>
+        <v>69.85999999999997</v>
       </c>
       <c r="K15" t="n">
-        <v>3.359999999999502</v>
+        <v>3.359999999999971</v>
       </c>
       <c r="L15" t="n">
-        <v>76.03999999999951</v>
+        <v>76.03999999999996</v>
       </c>
       <c r="M15" t="n">
-        <v>78.2199999999995</v>
+        <v>78.21999999999997</v>
       </c>
       <c r="N15" t="n">
-        <v>76.03999999999951</v>
+        <v>76.03999999999996</v>
       </c>
     </row>
     <row r="16">
@@ -1211,13 +1211,13 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>77.67999999999944</v>
+        <v>77.67999999999967</v>
       </c>
       <c r="M16" t="n">
-        <v>79.85999999999945</v>
+        <v>79.85999999999967</v>
       </c>
       <c r="N16" t="n">
-        <v>77.67999999999944</v>
+        <v>77.67999999999967</v>
       </c>
     </row>
     <row r="17">
@@ -1253,19 +1253,19 @@
         <v>76.5</v>
       </c>
       <c r="J17" t="n">
-        <v>79.85999999999945</v>
+        <v>79.85999999999962</v>
       </c>
       <c r="K17" t="n">
-        <v>3.359999999999445</v>
+        <v>3.359999999999616</v>
       </c>
       <c r="L17" t="n">
-        <v>86.03999999999945</v>
+        <v>86.03999999999962</v>
       </c>
       <c r="M17" t="n">
-        <v>88.21999999999944</v>
+        <v>88.21999999999962</v>
       </c>
       <c r="N17" t="n">
-        <v>86.03999999999945</v>
+        <v>86.03999999999962</v>
       </c>
     </row>
     <row r="18">
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H18" t="n">
         <v>80</v>
@@ -1301,19 +1301,19 @@
         <v>81.5</v>
       </c>
       <c r="J18" t="n">
-        <v>81.5</v>
+        <v>88.21999999999963</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>6.719999999999629</v>
       </c>
       <c r="L18" t="n">
-        <v>87.80999999999943</v>
+        <v>94.52999999999963</v>
       </c>
       <c r="M18" t="n">
-        <v>90.12999999999943</v>
+        <v>96.84999999999999</v>
       </c>
       <c r="N18" t="n">
-        <v>87.80999999999943</v>
+        <v>94.52999999999963</v>
       </c>
     </row>
     <row r="19">
@@ -1349,19 +1349,19 @@
         <v>86.5</v>
       </c>
       <c r="J19" t="n">
-        <v>90.12999999999931</v>
+        <v>86.5</v>
       </c>
       <c r="K19" t="n">
-        <v>3.629999999999313</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>96.43999999999932</v>
+        <v>92.80999999999989</v>
       </c>
       <c r="M19" t="n">
-        <v>98.75999999999931</v>
+        <v>95.12999999999988</v>
       </c>
       <c r="N19" t="n">
-        <v>96.43999999999932</v>
+        <v>92.80999999999989</v>
       </c>
     </row>
     <row r="20">
@@ -1397,19 +1397,19 @@
         <v>91.5</v>
       </c>
       <c r="J20" t="n">
-        <v>98.75999999999931</v>
+        <v>95.12999999999988</v>
       </c>
       <c r="K20" t="n">
-        <v>7.259999999999309</v>
+        <v>3.629999999999882</v>
       </c>
       <c r="L20" t="n">
-        <v>105.0699999999993</v>
+        <v>101.4399999999999</v>
       </c>
       <c r="M20" t="n">
-        <v>107.3899999999993</v>
+        <v>103.7599999999999</v>
       </c>
       <c r="N20" t="n">
-        <v>105.0699999999993</v>
+        <v>101.4399999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1445,19 +1445,19 @@
         <v>96.5</v>
       </c>
       <c r="J21" t="n">
-        <v>107.3899999999993</v>
+        <v>103.7599999999999</v>
       </c>
       <c r="K21" t="n">
-        <v>10.8899999999993</v>
+        <v>7.259999999999877</v>
       </c>
       <c r="L21" t="n">
-        <v>113.7</v>
+        <v>110.0699999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>116.0199999999993</v>
+        <v>112.3899999999999</v>
       </c>
       <c r="N21" t="n">
-        <v>113.7</v>
+        <v>110.0699999999999</v>
       </c>
     </row>
     <row r="22">
@@ -1499,13 +1499,13 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>107.8099999999994</v>
+        <v>107.8099999999999</v>
       </c>
       <c r="M22" t="n">
-        <v>110.1299999999994</v>
+        <v>110.1299999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>107.8099999999994</v>
+        <v>107.8099999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1541,19 +1541,19 @@
         <v>106.5</v>
       </c>
       <c r="J23" t="n">
-        <v>110.1299999999994</v>
+        <v>110.1299999999999</v>
       </c>
       <c r="K23" t="n">
-        <v>3.629999999999427</v>
+        <v>3.629999999999882</v>
       </c>
       <c r="L23" t="n">
-        <v>116.4399999999994</v>
+        <v>116.4399999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>118.7599999999994</v>
+        <v>118.7599999999999</v>
       </c>
       <c r="N23" t="n">
-        <v>116.4399999999994</v>
+        <v>116.4399999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1589,19 +1589,19 @@
         <v>111.5</v>
       </c>
       <c r="J24" t="n">
-        <v>118.7599999999994</v>
+        <v>118.7599999999998</v>
       </c>
       <c r="K24" t="n">
-        <v>7.259999999999422</v>
+        <v>7.25999999999982</v>
       </c>
       <c r="L24" t="n">
-        <v>125.0699999999994</v>
+        <v>125.0699999999998</v>
       </c>
       <c r="M24" t="n">
-        <v>127.3899999999994</v>
+        <v>127.3899999999998</v>
       </c>
       <c r="N24" t="n">
-        <v>125.0699999999994</v>
+        <v>125.0699999999998</v>
       </c>
     </row>
     <row r="25">
@@ -1625,10 +1625,10 @@
         <v>23</v>
       </c>
       <c r="F25" t="n">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
         <v>115</v>
@@ -1637,19 +1637,19 @@
         <v>116.5</v>
       </c>
       <c r="J25" t="n">
-        <v>127.3899999999994</v>
+        <v>116.5</v>
       </c>
       <c r="K25" t="n">
-        <v>10.88999999999942</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>133.7</v>
+        <v>122.8099999999999</v>
       </c>
       <c r="M25" t="n">
-        <v>136.0199999999994</v>
+        <v>125.1299999999999</v>
       </c>
       <c r="N25" t="n">
-        <v>133.7</v>
+        <v>122.8099999999999</v>
       </c>
     </row>
     <row r="26">
@@ -1685,19 +1685,19 @@
         <v>121.5</v>
       </c>
       <c r="J26" t="n">
-        <v>121.5</v>
+        <v>125.1299999999999</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>3.629999999999939</v>
       </c>
       <c r="L26" t="n">
-        <v>128.0099999999994</v>
+        <v>131.6399999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>130.5299999999994</v>
+        <v>134.1599999999999</v>
       </c>
       <c r="N26" t="n">
-        <v>128.0099999999994</v>
+        <v>131.6399999999999</v>
       </c>
     </row>
     <row r="27">
@@ -1733,19 +1733,19 @@
         <v>126.5</v>
       </c>
       <c r="J27" t="n">
-        <v>130.5299999999993</v>
+        <v>134.1599999999999</v>
       </c>
       <c r="K27" t="n">
-        <v>4.029999999999291</v>
+        <v>7.65999999999994</v>
       </c>
       <c r="L27" t="n">
-        <v>137.0399999999993</v>
+        <v>140.6699999999999</v>
       </c>
       <c r="M27" t="n">
-        <v>139.5599999999993</v>
+        <v>143.1899999999999</v>
       </c>
       <c r="N27" t="n">
-        <v>137.0399999999993</v>
+        <v>140.6699999999999</v>
       </c>
     </row>
     <row r="28">
@@ -1781,19 +1781,19 @@
         <v>131.5</v>
       </c>
       <c r="J28" t="n">
-        <v>139.5599999999993</v>
+        <v>143.1899999999999</v>
       </c>
       <c r="K28" t="n">
-        <v>8.059999999999263</v>
+        <v>11.68999999999994</v>
       </c>
       <c r="L28" t="n">
-        <v>146.0699999999993</v>
+        <v>149.7</v>
       </c>
       <c r="M28" t="n">
-        <v>148.5899999999993</v>
+        <v>152.2199999999999</v>
       </c>
       <c r="N28" t="n">
-        <v>146.0699999999993</v>
+        <v>149.7</v>
       </c>
     </row>
     <row r="29">
@@ -1817,7 +1817,7 @@
         <v>27</v>
       </c>
       <c r="F29" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="G29" t="n">
         <v>3</v>
@@ -1835,13 +1835,13 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>143.0099999999995</v>
+        <v>143.0099999999999</v>
       </c>
       <c r="M29" t="n">
-        <v>145.5299999999995</v>
+        <v>145.5299999999999</v>
       </c>
       <c r="N29" t="n">
-        <v>143.0099999999995</v>
+        <v>143.0099999999999</v>
       </c>
     </row>
     <row r="30">
@@ -1865,7 +1865,7 @@
         <v>28</v>
       </c>
       <c r="F30" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G30" t="n">
         <v>3</v>
@@ -1877,19 +1877,19 @@
         <v>141.5</v>
       </c>
       <c r="J30" t="n">
-        <v>145.5299999999994</v>
+        <v>145.5299999999999</v>
       </c>
       <c r="K30" t="n">
-        <v>4.029999999999404</v>
+        <v>4.029999999999944</v>
       </c>
       <c r="L30" t="n">
-        <v>152.0399999999994</v>
+        <v>152.0399999999999</v>
       </c>
       <c r="M30" t="n">
-        <v>154.5599999999994</v>
+        <v>154.5599999999999</v>
       </c>
       <c r="N30" t="n">
-        <v>152.0399999999994</v>
+        <v>152.0399999999999</v>
       </c>
     </row>
     <row r="31">
@@ -1925,16 +1925,16 @@
         <v>146.5</v>
       </c>
       <c r="J31" t="n">
-        <v>154.5599999999994</v>
+        <v>154.5599999999999</v>
       </c>
       <c r="K31" t="n">
-        <v>8.059999999999377</v>
+        <v>8.059999999999945</v>
       </c>
       <c r="L31" t="n">
-        <v>161.0699999999994</v>
+        <v>161.0699999999999</v>
       </c>
       <c r="M31" t="n">
-        <v>163.5899999999994</v>
+        <v>163.5899999999999</v>
       </c>
       <c r="N31" t="n">
         <v>170.1</v>
@@ -1973,16 +1973,16 @@
         <v>151.5</v>
       </c>
       <c r="J32" t="n">
-        <v>163.5899999999993</v>
+        <v>163.5899999999999</v>
       </c>
       <c r="K32" t="n">
-        <v>12.08999999999935</v>
+        <v>12.08999999999995</v>
       </c>
       <c r="L32" t="n">
         <v>170.1</v>
       </c>
       <c r="M32" t="n">
-        <v>172.6199999999994</v>
+        <v>172.6199999999999</v>
       </c>
       <c r="N32" t="n">
         <v>170.1</v>
@@ -2027,13 +2027,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>163.3899999999995</v>
+        <v>163.3899999999999</v>
       </c>
       <c r="M33" t="n">
-        <v>164.7199999999995</v>
+        <v>164.7199999999999</v>
       </c>
       <c r="N33" t="n">
-        <v>163.3899999999995</v>
+        <v>163.3899999999999</v>
       </c>
     </row>
     <row r="34">
@@ -2075,13 +2075,13 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>168.3899999999988</v>
+        <v>168.3899999999983</v>
       </c>
       <c r="M34" t="n">
-        <v>169.7199999999988</v>
+        <v>169.7199999999983</v>
       </c>
       <c r="N34" t="n">
-        <v>175.0599999999988</v>
+        <v>175.0599999999983</v>
       </c>
     </row>
     <row r="35">
@@ -2117,19 +2117,19 @@
         <v>168.05</v>
       </c>
       <c r="J35" t="n">
-        <v>169.7199999999988</v>
+        <v>169.7199999999983</v>
       </c>
       <c r="K35" t="n">
-        <v>1.669999999998822</v>
+        <v>1.669999999998311</v>
       </c>
       <c r="L35" t="n">
-        <v>175.0599999999988</v>
+        <v>175.0599999999983</v>
       </c>
       <c r="M35" t="n">
-        <v>176.3899999999988</v>
+        <v>176.3899999999983</v>
       </c>
       <c r="N35" t="n">
-        <v>175.0599999999988</v>
+        <v>175.0599999999983</v>
       </c>
     </row>
     <row r="36">
@@ -2171,13 +2171,13 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>178.5599999999988</v>
+        <v>178.5599999999981</v>
       </c>
       <c r="M36" t="n">
-        <v>180.0799999999988</v>
+        <v>180.0799999999981</v>
       </c>
       <c r="N36" t="n">
-        <v>185.5899999999988</v>
+        <v>185.5899999999981</v>
       </c>
     </row>
     <row r="37">
@@ -2213,19 +2213,19 @@
         <v>178.05</v>
       </c>
       <c r="J37" t="n">
-        <v>180.0799999999988</v>
+        <v>180.0799999999981</v>
       </c>
       <c r="K37" t="n">
-        <v>2.029999999998779</v>
+        <v>2.029999999998097</v>
       </c>
       <c r="L37" t="n">
-        <v>185.5899999999988</v>
+        <v>185.5899999999981</v>
       </c>
       <c r="M37" t="n">
-        <v>187.1099999999988</v>
+        <v>187.1099999999981</v>
       </c>
       <c r="N37" t="n">
-        <v>185.5899999999988</v>
+        <v>185.5899999999981</v>
       </c>
     </row>
     <row r="38">
@@ -2267,13 +2267,13 @@
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>188.5599999999994</v>
+        <v>188.5599999999996</v>
       </c>
       <c r="M38" t="n">
-        <v>190.0799999999994</v>
+        <v>190.0799999999996</v>
       </c>
       <c r="N38" t="n">
-        <v>188.5599999999994</v>
+        <v>188.5599999999996</v>
       </c>
     </row>
     <row r="39">
@@ -2315,13 +2315,13 @@
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>193.8699999999994</v>
+        <v>193.8699999999996</v>
       </c>
       <c r="M39" t="n">
         <v>195.7</v>
       </c>
       <c r="N39" t="n">
-        <v>193.8699999999994</v>
+        <v>193.8699999999996</v>
       </c>
     </row>
     <row r="40">
@@ -2360,16 +2360,16 @@
         <v>195.7</v>
       </c>
       <c r="K40" t="n">
-        <v>2.649999999999977</v>
+        <v>2.65</v>
       </c>
       <c r="L40" t="n">
-        <v>201.5199999999994</v>
+        <v>201.5199999999996</v>
       </c>
       <c r="M40" t="n">
         <v>203.35</v>
       </c>
       <c r="N40" t="n">
-        <v>201.5199999999994</v>
+        <v>201.5199999999996</v>
       </c>
     </row>
     <row r="41">
@@ -2411,13 +2411,13 @@
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>203.8699999999994</v>
+        <v>203.8699999999991</v>
       </c>
       <c r="M41" t="n">
         <v>205.7</v>
       </c>
       <c r="N41" t="n">
-        <v>203.8699999999994</v>
+        <v>203.8699999999991</v>
       </c>
     </row>
     <row r="42">
@@ -2456,16 +2456,16 @@
         <v>205.7</v>
       </c>
       <c r="K42" t="n">
-        <v>2.649999999999977</v>
+        <v>2.65</v>
       </c>
       <c r="L42" t="n">
-        <v>211.5199999999994</v>
+        <v>211.5199999999991</v>
       </c>
       <c r="M42" t="n">
         <v>213.35</v>
       </c>
       <c r="N42" t="n">
-        <v>211.5199999999994</v>
+        <v>211.5199999999991</v>
       </c>
     </row>
     <row r="43">
@@ -2510,7 +2510,7 @@
         <v>213.9</v>
       </c>
       <c r="M43" t="n">
-        <v>215.7399999999993</v>
+        <v>215.739999999999</v>
       </c>
       <c r="N43" t="n">
         <v>213.9</v>
@@ -2549,19 +2549,19 @@
         <v>213.05</v>
       </c>
       <c r="J44" t="n">
-        <v>215.7399999999993</v>
+        <v>215.7399999999968</v>
       </c>
       <c r="K44" t="n">
-        <v>2.689999999999259</v>
+        <v>2.689999999996758</v>
       </c>
       <c r="L44" t="n">
-        <v>221.5899999999993</v>
+        <v>221.5899999999968</v>
       </c>
       <c r="M44" t="n">
-        <v>223.4299999999993</v>
+        <v>223.4299999999968</v>
       </c>
       <c r="N44" t="n">
-        <v>221.5899999999993</v>
+        <v>221.5899999999968</v>
       </c>
     </row>
     <row r="45">
@@ -2606,7 +2606,7 @@
         <v>223.9</v>
       </c>
       <c r="M45" t="n">
-        <v>225.7399999999994</v>
+        <v>225.7399999999997</v>
       </c>
       <c r="N45" t="n">
         <v>223.9</v>
@@ -2645,19 +2645,19 @@
         <v>223.05</v>
       </c>
       <c r="J46" t="n">
-        <v>225.7399999999994</v>
+        <v>225.7399999999997</v>
       </c>
       <c r="K46" t="n">
-        <v>2.689999999999429</v>
+        <v>2.689999999999657</v>
       </c>
       <c r="L46" t="n">
-        <v>231.5899999999994</v>
+        <v>231.5899999999997</v>
       </c>
       <c r="M46" t="n">
-        <v>233.4299999999994</v>
+        <v>233.4299999999997</v>
       </c>
       <c r="N46" t="n">
-        <v>231.5899999999994</v>
+        <v>231.5899999999997</v>
       </c>
     </row>
     <row r="47">
@@ -2699,13 +2699,13 @@
         <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>234.2299999999985</v>
+        <v>234.2299999999989</v>
       </c>
       <c r="M47" t="n">
-        <v>236.4099999999985</v>
+        <v>236.4099999999989</v>
       </c>
       <c r="N47" t="n">
-        <v>234.2299999999985</v>
+        <v>234.2299999999989</v>
       </c>
     </row>
     <row r="48">
@@ -2741,19 +2741,19 @@
         <v>233.05</v>
       </c>
       <c r="J48" t="n">
-        <v>236.4099999999985</v>
+        <v>236.4099999999989</v>
       </c>
       <c r="K48" t="n">
-        <v>3.359999999998536</v>
+        <v>3.359999999998877</v>
       </c>
       <c r="L48" t="n">
-        <v>242.5899999999986</v>
+        <v>242.5899999999989</v>
       </c>
       <c r="M48" t="n">
-        <v>244.7699999999986</v>
+        <v>244.7699999999989</v>
       </c>
       <c r="N48" t="n">
-        <v>242.5899999999986</v>
+        <v>242.5899999999989</v>
       </c>
     </row>
     <row r="49">
@@ -2795,13 +2795,13 @@
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>244.2299999999994</v>
+        <v>244.2299999999997</v>
       </c>
       <c r="M49" t="n">
-        <v>246.4099999999995</v>
+        <v>246.4099999999997</v>
       </c>
       <c r="N49" t="n">
-        <v>244.2299999999994</v>
+        <v>244.2299999999997</v>
       </c>
     </row>
     <row r="50">
@@ -2837,19 +2837,19 @@
         <v>243.05</v>
       </c>
       <c r="J50" t="n">
-        <v>246.4099999999995</v>
+        <v>246.4099999999997</v>
       </c>
       <c r="K50" t="n">
-        <v>3.359999999999445</v>
+        <v>3.359999999999673</v>
       </c>
       <c r="L50" t="n">
-        <v>252.5899999999995</v>
+        <v>252.5899999999997</v>
       </c>
       <c r="M50" t="n">
-        <v>254.7699999999995</v>
+        <v>254.7699999999997</v>
       </c>
       <c r="N50" t="n">
-        <v>252.5899999999995</v>
+        <v>252.5899999999997</v>
       </c>
     </row>
     <row r="51">
@@ -2933,19 +2933,19 @@
         <v>253.05</v>
       </c>
       <c r="J52" t="n">
-        <v>256.6799999999993</v>
+        <v>256.6799999999994</v>
       </c>
       <c r="K52" t="n">
-        <v>3.629999999999256</v>
+        <v>3.629999999999427</v>
       </c>
       <c r="L52" t="n">
-        <v>262.9899999999993</v>
+        <v>262.9899999999994</v>
       </c>
       <c r="M52" t="n">
-        <v>265.3099999999993</v>
+        <v>265.3099999999994</v>
       </c>
       <c r="N52" t="n">
-        <v>271.6199999999993</v>
+        <v>271.6199999999994</v>
       </c>
     </row>
     <row r="53">
@@ -2981,19 +2981,19 @@
         <v>258.05</v>
       </c>
       <c r="J53" t="n">
-        <v>265.3099999999993</v>
+        <v>265.3099999999994</v>
       </c>
       <c r="K53" t="n">
-        <v>7.259999999999252</v>
+        <v>7.259999999999422</v>
       </c>
       <c r="L53" t="n">
-        <v>271.6199999999993</v>
+        <v>271.6199999999994</v>
       </c>
       <c r="M53" t="n">
-        <v>273.9399999999993</v>
+        <v>273.9399999999994</v>
       </c>
       <c r="N53" t="n">
-        <v>271.6199999999993</v>
+        <v>271.6199999999994</v>
       </c>
     </row>
     <row r="54">
@@ -3029,16 +3029,16 @@
         <v>263.05</v>
       </c>
       <c r="J54" t="n">
-        <v>273.9399999999993</v>
+        <v>273.9399999999994</v>
       </c>
       <c r="K54" t="n">
-        <v>10.88999999999925</v>
+        <v>10.88999999999942</v>
       </c>
       <c r="L54" t="n">
         <v>280.25</v>
       </c>
       <c r="M54" t="n">
-        <v>282.5699999999993</v>
+        <v>282.5699999999994</v>
       </c>
       <c r="N54" t="n">
         <v>280.25</v>
@@ -3077,19 +3077,19 @@
         <v>268.05</v>
       </c>
       <c r="J55" t="n">
-        <v>282.5699999999993</v>
+        <v>282.5699999999994</v>
       </c>
       <c r="K55" t="n">
-        <v>14.51999999999924</v>
+        <v>14.51999999999941</v>
       </c>
       <c r="L55" t="n">
-        <v>288.8799999999993</v>
+        <v>288.8799999999994</v>
       </c>
       <c r="M55" t="n">
         <v>291.2</v>
       </c>
       <c r="N55" t="n">
-        <v>288.8799999999993</v>
+        <v>288.8799999999994</v>
       </c>
     </row>
     <row r="56">
@@ -3131,13 +3131,13 @@
         <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>279.3599999999996</v>
+        <v>279.359999999999</v>
       </c>
       <c r="M56" t="n">
-        <v>281.6799999999996</v>
+        <v>281.679999999999</v>
       </c>
       <c r="N56" t="n">
-        <v>279.3599999999996</v>
+        <v>279.359999999999</v>
       </c>
     </row>
     <row r="57">
@@ -3173,19 +3173,19 @@
         <v>278.05</v>
       </c>
       <c r="J57" t="n">
-        <v>281.6799999999994</v>
+        <v>281.679999999999</v>
       </c>
       <c r="K57" t="n">
-        <v>3.629999999999427</v>
+        <v>3.629999999998972</v>
       </c>
       <c r="L57" t="n">
-        <v>287.9899999999994</v>
+        <v>287.989999999999</v>
       </c>
       <c r="M57" t="n">
-        <v>290.3099999999994</v>
+        <v>290.309999999999</v>
       </c>
       <c r="N57" t="n">
-        <v>287.9899999999994</v>
+        <v>287.989999999999</v>
       </c>
     </row>
     <row r="58">
@@ -3221,19 +3221,19 @@
         <v>283.05</v>
       </c>
       <c r="J58" t="n">
-        <v>290.3099999999994</v>
+        <v>290.309999999999</v>
       </c>
       <c r="K58" t="n">
-        <v>7.259999999999422</v>
+        <v>7.259999999998968</v>
       </c>
       <c r="L58" t="n">
-        <v>296.6199999999994</v>
+        <v>296.619999999999</v>
       </c>
       <c r="M58" t="n">
-        <v>298.9399999999994</v>
+        <v>298.939999999999</v>
       </c>
       <c r="N58" t="n">
-        <v>296.6199999999994</v>
+        <v>296.619999999999</v>
       </c>
     </row>
     <row r="59">
@@ -3269,16 +3269,16 @@
         <v>288.05</v>
       </c>
       <c r="J59" t="n">
-        <v>298.9399999999994</v>
+        <v>298.939999999999</v>
       </c>
       <c r="K59" t="n">
-        <v>10.88999999999942</v>
+        <v>10.88999999999896</v>
       </c>
       <c r="L59" t="n">
         <v>305.25</v>
       </c>
       <c r="M59" t="n">
-        <v>307.5699999999994</v>
+        <v>307.569999999999</v>
       </c>
       <c r="N59" t="n">
         <v>305.25</v>
@@ -3323,13 +3323,13 @@
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>299.5599999999995</v>
+        <v>299.5599999999997</v>
       </c>
       <c r="M60" t="n">
-        <v>302.0799999999996</v>
+        <v>302.0799999999997</v>
       </c>
       <c r="N60" t="n">
-        <v>299.5599999999995</v>
+        <v>299.5599999999997</v>
       </c>
     </row>
     <row r="61">
@@ -3353,7 +3353,7 @@
         <v>59</v>
       </c>
       <c r="F61" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G61" t="n">
         <v>1</v>
@@ -3365,19 +3365,19 @@
         <v>298.05</v>
       </c>
       <c r="J61" t="n">
-        <v>302.0799999999984</v>
+        <v>302.0799999999997</v>
       </c>
       <c r="K61" t="n">
-        <v>4.029999999998381</v>
+        <v>4.029999999999688</v>
       </c>
       <c r="L61" t="n">
-        <v>308.5899999999984</v>
+        <v>308.5899999999997</v>
       </c>
       <c r="M61" t="n">
-        <v>311.1099999999984</v>
+        <v>311.1099999999997</v>
       </c>
       <c r="N61" t="n">
-        <v>308.5899999999984</v>
+        <v>308.5899999999997</v>
       </c>
     </row>
     <row r="62">
@@ -3401,7 +3401,7 @@
         <v>60</v>
       </c>
       <c r="F62" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
@@ -3413,19 +3413,19 @@
         <v>303.05</v>
       </c>
       <c r="J62" t="n">
-        <v>311.1099999999984</v>
+        <v>311.1099999999997</v>
       </c>
       <c r="K62" t="n">
-        <v>8.059999999998411</v>
+        <v>8.059999999999661</v>
       </c>
       <c r="L62" t="n">
-        <v>317.6199999999984</v>
+        <v>317.6199999999997</v>
       </c>
       <c r="M62" t="n">
-        <v>320.1399999999984</v>
+        <v>320.1399999999996</v>
       </c>
       <c r="N62" t="n">
-        <v>317.6199999999984</v>
+        <v>317.6199999999997</v>
       </c>
     </row>
     <row r="63">
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>314.5599999999994</v>
+        <v>314.5599999999996</v>
       </c>
       <c r="M63" t="n">
-        <v>317.0799999999994</v>
+        <v>317.0799999999996</v>
       </c>
       <c r="N63" t="n">
-        <v>314.5599999999994</v>
+        <v>314.5599999999996</v>
       </c>
     </row>
     <row r="64">
@@ -3509,19 +3509,19 @@
         <v>313.05</v>
       </c>
       <c r="J64" t="n">
-        <v>317.0799999999992</v>
+        <v>317.0799999999996</v>
       </c>
       <c r="K64" t="n">
-        <v>4.029999999999234</v>
+        <v>4.029999999999575</v>
       </c>
       <c r="L64" t="n">
-        <v>323.5899999999992</v>
+        <v>323.5899999999996</v>
       </c>
       <c r="M64" t="n">
-        <v>326.1099999999992</v>
+        <v>326.1099999999996</v>
       </c>
       <c r="N64" t="n">
-        <v>323.5899999999992</v>
+        <v>323.5899999999996</v>
       </c>
     </row>
     <row r="65">
@@ -3557,19 +3557,19 @@
         <v>318.05</v>
       </c>
       <c r="J65" t="n">
-        <v>326.1099999999992</v>
+        <v>326.1099999999996</v>
       </c>
       <c r="K65" t="n">
-        <v>8.059999999999206</v>
+        <v>8.059999999999548</v>
       </c>
       <c r="L65" t="n">
-        <v>332.6199999999992</v>
+        <v>332.6199999999995</v>
       </c>
       <c r="M65" t="n">
-        <v>335.1399999999992</v>
+        <v>335.1399999999995</v>
       </c>
       <c r="N65" t="n">
-        <v>332.6199999999992</v>
+        <v>332.6199999999995</v>
       </c>
     </row>
     <row r="66">
@@ -3611,13 +3611,13 @@
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>329.9399999999989</v>
+        <v>329.9399999999999</v>
       </c>
       <c r="M66" t="n">
-        <v>331.269999999999</v>
+        <v>331.2699999999999</v>
       </c>
       <c r="N66" t="n">
-        <v>329.9399999999989</v>
+        <v>329.9399999999999</v>
       </c>
     </row>
     <row r="67">
@@ -3659,13 +3659,13 @@
         <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>334.9399999999989</v>
+        <v>334.9399999999999</v>
       </c>
       <c r="M67" t="n">
-        <v>336.269999999999</v>
+        <v>336.2699999999999</v>
       </c>
       <c r="N67" t="n">
-        <v>334.9399999999989</v>
+        <v>334.9399999999999</v>
       </c>
     </row>
     <row r="68">
@@ -3707,13 +3707,13 @@
         <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>340.1099999999982</v>
+        <v>340.1099999999999</v>
       </c>
       <c r="M68" t="n">
-        <v>341.6299999999982</v>
+        <v>341.6299999999999</v>
       </c>
       <c r="N68" t="n">
-        <v>340.1099999999982</v>
+        <v>340.1099999999999</v>
       </c>
     </row>
     <row r="69">
@@ -3755,13 +3755,13 @@
         <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>345.1099999999994</v>
+        <v>345.1099999999999</v>
       </c>
       <c r="M69" t="n">
-        <v>346.6299999999994</v>
+        <v>346.6299999999999</v>
       </c>
       <c r="N69" t="n">
-        <v>345.1099999999994</v>
+        <v>345.1099999999999</v>
       </c>
     </row>
     <row r="70">
@@ -3803,13 +3803,13 @@
         <v>0</v>
       </c>
       <c r="L70" t="n">
-        <v>350.4199999999988</v>
+        <v>350.4199999999997</v>
       </c>
       <c r="M70" t="n">
         <v>352.25</v>
       </c>
       <c r="N70" t="n">
-        <v>350.4199999999988</v>
+        <v>350.4199999999997</v>
       </c>
     </row>
     <row r="71">
@@ -3848,16 +3848,16 @@
         <v>352.25</v>
       </c>
       <c r="K71" t="n">
-        <v>2.649999999999977</v>
+        <v>2.65</v>
       </c>
       <c r="L71" t="n">
-        <v>358.0699999999956</v>
+        <v>358.0699999999995</v>
       </c>
       <c r="M71" t="n">
         <v>359.9</v>
       </c>
       <c r="N71" t="n">
-        <v>358.0699999999956</v>
+        <v>358.0699999999995</v>
       </c>
     </row>
     <row r="72">
@@ -3899,13 +3899,13 @@
         <v>0</v>
       </c>
       <c r="L72" t="n">
-        <v>360.4199999999985</v>
+        <v>360.42</v>
       </c>
       <c r="M72" t="n">
         <v>362.25</v>
       </c>
       <c r="N72" t="n">
-        <v>360.4199999999985</v>
+        <v>360.42</v>
       </c>
     </row>
     <row r="73">
@@ -3944,16 +3944,16 @@
         <v>362.25</v>
       </c>
       <c r="K73" t="n">
-        <v>2.649999999999977</v>
+        <v>2.65</v>
       </c>
       <c r="L73" t="n">
-        <v>368.0699999999964</v>
+        <v>368.0699999999999</v>
       </c>
       <c r="M73" t="n">
         <v>369.9</v>
       </c>
       <c r="N73" t="n">
-        <v>368.0699999999964</v>
+        <v>368.0699999999999</v>
       </c>
     </row>
     <row r="74">
@@ -3998,7 +3998,7 @@
         <v>370.45</v>
       </c>
       <c r="M74" t="n">
-        <v>372.2899999999983</v>
+        <v>372.2899999999997</v>
       </c>
       <c r="N74" t="n">
         <v>370.45</v>
@@ -4037,19 +4037,19 @@
         <v>369.6</v>
       </c>
       <c r="J75" t="n">
-        <v>372.2899999999965</v>
+        <v>372.2899999999993</v>
       </c>
       <c r="K75" t="n">
-        <v>2.689999999996473</v>
+        <v>2.689999999999316</v>
       </c>
       <c r="L75" t="n">
-        <v>378.1399999999965</v>
+        <v>378.1399999999994</v>
       </c>
       <c r="M75" t="n">
-        <v>379.9799999999965</v>
+        <v>379.9799999999993</v>
       </c>
       <c r="N75" t="n">
-        <v>378.1399999999965</v>
+        <v>378.1399999999994</v>
       </c>
     </row>
     <row r="76">
@@ -4094,7 +4094,7 @@
         <v>380.45</v>
       </c>
       <c r="M76" t="n">
-        <v>382.2899999999985</v>
+        <v>382.2899999999997</v>
       </c>
       <c r="N76" t="n">
         <v>380.45</v>
@@ -4133,19 +4133,19 @@
         <v>379.6</v>
       </c>
       <c r="J77" t="n">
-        <v>382.2899999999952</v>
+        <v>382.2899999999996</v>
       </c>
       <c r="K77" t="n">
-        <v>2.689999999995223</v>
+        <v>2.6899999999996</v>
       </c>
       <c r="L77" t="n">
-        <v>388.1399999999953</v>
+        <v>388.1399999999996</v>
       </c>
       <c r="M77" t="n">
-        <v>389.9799999999952</v>
+        <v>389.9799999999996</v>
       </c>
       <c r="N77" t="n">
-        <v>388.1399999999953</v>
+        <v>388.1399999999996</v>
       </c>
     </row>
     <row r="78">
@@ -4187,13 +4187,13 @@
         <v>0</v>
       </c>
       <c r="L78" t="n">
-        <v>390.779999999998</v>
+        <v>390.7799999999997</v>
       </c>
       <c r="M78" t="n">
-        <v>392.959999999998</v>
+        <v>392.9599999999997</v>
       </c>
       <c r="N78" t="n">
-        <v>390.779999999998</v>
+        <v>390.7799999999997</v>
       </c>
     </row>
     <row r="79">
@@ -4229,19 +4229,19 @@
         <v>389.6</v>
       </c>
       <c r="J79" t="n">
-        <v>392.9599999999962</v>
+        <v>392.9599999999997</v>
       </c>
       <c r="K79" t="n">
-        <v>3.359999999996148</v>
+        <v>3.359999999999673</v>
       </c>
       <c r="L79" t="n">
-        <v>399.1399999999962</v>
+        <v>399.1399999999997</v>
       </c>
       <c r="M79" t="n">
-        <v>401.3199999999962</v>
+        <v>401.3199999999997</v>
       </c>
       <c r="N79" t="n">
-        <v>399.1399999999962</v>
+        <v>399.1399999999997</v>
       </c>
     </row>
     <row r="80">
@@ -4283,13 +4283,13 @@
         <v>0</v>
       </c>
       <c r="L80" t="n">
-        <v>400.7799999999984</v>
+        <v>400.7799999999996</v>
       </c>
       <c r="M80" t="n">
-        <v>402.9599999999984</v>
+        <v>402.9599999999996</v>
       </c>
       <c r="N80" t="n">
-        <v>400.7799999999984</v>
+        <v>400.7799999999996</v>
       </c>
     </row>
     <row r="81">
@@ -4325,19 +4325,19 @@
         <v>399.6</v>
       </c>
       <c r="J81" t="n">
-        <v>402.9599999999949</v>
+        <v>402.9599999999992</v>
       </c>
       <c r="K81" t="n">
-        <v>3.359999999994898</v>
+        <v>3.359999999999218</v>
       </c>
       <c r="L81" t="n">
-        <v>409.1399999999949</v>
+        <v>409.1399999999992</v>
       </c>
       <c r="M81" t="n">
-        <v>411.3199999999949</v>
+        <v>411.3199999999993</v>
       </c>
       <c r="N81" t="n">
-        <v>409.1399999999949</v>
+        <v>409.1399999999992</v>
       </c>
     </row>
     <row r="82">
@@ -4379,13 +4379,13 @@
         <v>0</v>
       </c>
       <c r="L82" t="n">
-        <v>410.909999999998</v>
+        <v>410.9099999999995</v>
       </c>
       <c r="M82" t="n">
-        <v>413.229999999998</v>
+        <v>413.2299999999995</v>
       </c>
       <c r="N82" t="n">
-        <v>410.909999999998</v>
+        <v>410.9099999999995</v>
       </c>
     </row>
     <row r="83">
@@ -4421,19 +4421,19 @@
         <v>409.6</v>
       </c>
       <c r="J83" t="n">
-        <v>413.229999999996</v>
+        <v>413.2299999999993</v>
       </c>
       <c r="K83" t="n">
-        <v>3.629999999996016</v>
+        <v>3.629999999999256</v>
       </c>
       <c r="L83" t="n">
-        <v>419.539999999996</v>
+        <v>419.5399999999993</v>
       </c>
       <c r="M83" t="n">
-        <v>421.859999999996</v>
+        <v>421.8599999999993</v>
       </c>
       <c r="N83" t="n">
-        <v>419.539999999996</v>
+        <v>419.5399999999993</v>
       </c>
     </row>
     <row r="84">
@@ -4469,19 +4469,19 @@
         <v>414.6</v>
       </c>
       <c r="J84" t="n">
-        <v>421.8599999999959</v>
+        <v>421.859999999999</v>
       </c>
       <c r="K84" t="n">
-        <v>7.259999999995898</v>
+        <v>7.259999999999025</v>
       </c>
       <c r="L84" t="n">
-        <v>428.1699999999959</v>
+        <v>428.169999999999</v>
       </c>
       <c r="M84" t="n">
-        <v>430.4899999999959</v>
+        <v>430.489999999999</v>
       </c>
       <c r="N84" t="n">
-        <v>428.1699999999959</v>
+        <v>428.169999999999</v>
       </c>
     </row>
     <row r="85">
@@ -4517,16 +4517,16 @@
         <v>419.6</v>
       </c>
       <c r="J85" t="n">
-        <v>430.4899999999959</v>
+        <v>430.489999999999</v>
       </c>
       <c r="K85" t="n">
-        <v>10.88999999999589</v>
+        <v>10.88999999999902</v>
       </c>
       <c r="L85" t="n">
         <v>436.8</v>
       </c>
       <c r="M85" t="n">
-        <v>439.1199999999959</v>
+        <v>439.119999999999</v>
       </c>
       <c r="N85" t="n">
         <v>436.8</v>
@@ -4571,13 +4571,13 @@
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>430.9099999999978</v>
+        <v>430.9099999999997</v>
       </c>
       <c r="M86" t="n">
-        <v>433.2299999999977</v>
+        <v>433.2299999999997</v>
       </c>
       <c r="N86" t="n">
-        <v>430.9099999999978</v>
+        <v>430.9099999999997</v>
       </c>
     </row>
     <row r="87">
@@ -4613,19 +4613,19 @@
         <v>429.6</v>
       </c>
       <c r="J87" t="n">
-        <v>433.2299999999939</v>
+        <v>433.2299999999997</v>
       </c>
       <c r="K87" t="n">
-        <v>3.629999999993913</v>
+        <v>3.629999999999654</v>
       </c>
       <c r="L87" t="n">
-        <v>439.5399999999939</v>
+        <v>439.5399999999997</v>
       </c>
       <c r="M87" t="n">
-        <v>441.8599999999939</v>
+        <v>441.8599999999997</v>
       </c>
       <c r="N87" t="n">
-        <v>439.5399999999939</v>
+        <v>439.5399999999997</v>
       </c>
     </row>
     <row r="88">
@@ -4661,19 +4661,19 @@
         <v>434.6</v>
       </c>
       <c r="J88" t="n">
-        <v>441.8599999999911</v>
+        <v>441.8599999999989</v>
       </c>
       <c r="K88" t="n">
-        <v>7.259999999991123</v>
+        <v>7.259999999998854</v>
       </c>
       <c r="L88" t="n">
-        <v>448.1699999999911</v>
+        <v>448.1699999999989</v>
       </c>
       <c r="M88" t="n">
-        <v>450.4899999999911</v>
+        <v>450.4899999999989</v>
       </c>
       <c r="N88" t="n">
-        <v>448.1699999999911</v>
+        <v>448.1699999999989</v>
       </c>
     </row>
     <row r="89">
@@ -4709,16 +4709,16 @@
         <v>439.6</v>
       </c>
       <c r="J89" t="n">
-        <v>450.4899999999911</v>
+        <v>450.4899999999989</v>
       </c>
       <c r="K89" t="n">
-        <v>10.88999999999112</v>
+        <v>10.88999999999885</v>
       </c>
       <c r="L89" t="n">
         <v>456.8</v>
       </c>
       <c r="M89" t="n">
-        <v>459.1199999999911</v>
+        <v>459.1199999999989</v>
       </c>
       <c r="N89" t="n">
         <v>456.8</v>
@@ -4757,19 +4757,19 @@
         <v>444.6</v>
       </c>
       <c r="J90" t="n">
-        <v>459.1199999999911</v>
+        <v>459.1199999999983</v>
       </c>
       <c r="K90" t="n">
-        <v>14.51999999999111</v>
+        <v>14.51999999999828</v>
       </c>
       <c r="L90" t="n">
-        <v>465.6299999999911</v>
+        <v>465.6299999999983</v>
       </c>
       <c r="M90" t="n">
         <v>468.15</v>
       </c>
       <c r="N90" t="n">
-        <v>519.8099999999906</v>
+        <v>519.8099999999978</v>
       </c>
     </row>
     <row r="91">
@@ -4808,16 +4808,16 @@
         <v>468.15</v>
       </c>
       <c r="K91" t="n">
-        <v>18.54999999999995</v>
+        <v>18.55</v>
       </c>
       <c r="L91" t="n">
-        <v>474.6599999999911</v>
+        <v>474.6599999999983</v>
       </c>
       <c r="M91" t="n">
-        <v>477.1799999999911</v>
+        <v>477.1799999999982</v>
       </c>
       <c r="N91" t="n">
-        <v>528.8399999999906</v>
+        <v>528.8399999999973</v>
       </c>
     </row>
     <row r="92">
@@ -4853,16 +4853,16 @@
         <v>454.6</v>
       </c>
       <c r="J92" t="n">
-        <v>477.1799999999911</v>
+        <v>477.1799999999982</v>
       </c>
       <c r="K92" t="n">
-        <v>22.57999999999106</v>
+        <v>22.57999999999822</v>
       </c>
       <c r="L92" t="n">
-        <v>483.6899999999911</v>
+        <v>483.6899999999982</v>
       </c>
       <c r="M92" t="n">
-        <v>486.2099999999911</v>
+        <v>486.2099999999983</v>
       </c>
       <c r="N92" t="n">
         <v>546.9</v>
@@ -4907,13 +4907,13 @@
         <v>0</v>
       </c>
       <c r="L93" t="n">
-        <v>466.1099999999994</v>
+        <v>466.11</v>
       </c>
       <c r="M93" t="n">
-        <v>468.6299999999994</v>
+        <v>468.63</v>
       </c>
       <c r="N93" t="n">
-        <v>466.1099999999994</v>
+        <v>466.11</v>
       </c>
     </row>
     <row r="94">
@@ -4949,19 +4949,19 @@
         <v>464.6</v>
       </c>
       <c r="J94" t="n">
-        <v>468.629999999995</v>
+        <v>468.6299999999993</v>
       </c>
       <c r="K94" t="n">
-        <v>4.02999999999497</v>
+        <v>4.029999999999291</v>
       </c>
       <c r="L94" t="n">
-        <v>475.139999999995</v>
+        <v>475.1399999999993</v>
       </c>
       <c r="M94" t="n">
-        <v>477.659999999995</v>
+        <v>477.6599999999993</v>
       </c>
       <c r="N94" t="n">
-        <v>506.1099999999994</v>
+        <v>506.11</v>
       </c>
     </row>
     <row r="95">
@@ -4997,19 +4997,19 @@
         <v>469.6</v>
       </c>
       <c r="J95" t="n">
-        <v>477.659999999995</v>
+        <v>477.6599999999993</v>
       </c>
       <c r="K95" t="n">
-        <v>8.059999999994943</v>
+        <v>8.059999999999263</v>
       </c>
       <c r="L95" t="n">
-        <v>484.169999999995</v>
+        <v>484.1699999999993</v>
       </c>
       <c r="M95" t="n">
-        <v>486.6899999999949</v>
+        <v>486.6899999999993</v>
       </c>
       <c r="N95" t="n">
-        <v>515.1399999999983</v>
+        <v>515.14</v>
       </c>
     </row>
     <row r="96">
@@ -5045,19 +5045,19 @@
         <v>474.6</v>
       </c>
       <c r="J96" t="n">
-        <v>486.2099999999911</v>
+        <v>486.209999999998</v>
       </c>
       <c r="K96" t="n">
-        <v>11.60999999999103</v>
+        <v>11.60999999999797</v>
       </c>
       <c r="L96" t="n">
-        <v>492.719999999991</v>
+        <v>492.719999999998</v>
       </c>
       <c r="M96" t="n">
-        <v>495.239999999991</v>
+        <v>495.239999999998</v>
       </c>
       <c r="N96" t="n">
-        <v>519.8099999999906</v>
+        <v>519.8099999999978</v>
       </c>
     </row>
     <row r="97">
@@ -5093,19 +5093,19 @@
         <v>479.6</v>
       </c>
       <c r="J97" t="n">
-        <v>495.239999999991</v>
+        <v>495.239999999998</v>
       </c>
       <c r="K97" t="n">
-        <v>15.63999999999101</v>
+        <v>15.63999999999794</v>
       </c>
       <c r="L97" t="n">
         <v>501.75</v>
       </c>
       <c r="M97" t="n">
-        <v>504.269999999991</v>
+        <v>504.2699999999979</v>
       </c>
       <c r="N97" t="n">
-        <v>528.8399999999906</v>
+        <v>528.8399999999973</v>
       </c>
     </row>
     <row r="98">
@@ -5141,19 +5141,19 @@
         <v>484.6</v>
       </c>
       <c r="J98" t="n">
-        <v>504.269999999991</v>
+        <v>504.2699999999979</v>
       </c>
       <c r="K98" t="n">
-        <v>19.66999999999098</v>
+        <v>19.66999999999791</v>
       </c>
       <c r="L98" t="n">
-        <v>510.779999999991</v>
+        <v>510.7799999999979</v>
       </c>
       <c r="M98" t="n">
         <v>513.3</v>
       </c>
       <c r="N98" t="n">
-        <v>519.8099999999906</v>
+        <v>519.8099999999978</v>
       </c>
     </row>
     <row r="99">
@@ -5192,16 +5192,16 @@
         <v>513.3</v>
       </c>
       <c r="K99" t="n">
-        <v>23.69999999999993</v>
+        <v>23.7</v>
       </c>
       <c r="L99" t="n">
-        <v>519.809999999991</v>
+        <v>519.8099999999979</v>
       </c>
       <c r="M99" t="n">
-        <v>522.3299999999909</v>
+        <v>522.3299999999979</v>
       </c>
       <c r="N99" t="n">
-        <v>519.8099999999906</v>
+        <v>519.8099999999978</v>
       </c>
     </row>
     <row r="100">
@@ -5237,19 +5237,19 @@
         <v>494.6</v>
       </c>
       <c r="J100" t="n">
-        <v>522.3299999999909</v>
+        <v>522.3299999999979</v>
       </c>
       <c r="K100" t="n">
-        <v>27.72999999999092</v>
+        <v>27.72999999999786</v>
       </c>
       <c r="L100" t="n">
-        <v>528.8399999999909</v>
+        <v>528.8399999999979</v>
       </c>
       <c r="M100" t="n">
-        <v>531.3599999999909</v>
+        <v>531.3599999999979</v>
       </c>
       <c r="N100" t="n">
-        <v>528.8399999999906</v>
+        <v>528.8399999999973</v>
       </c>
     </row>
     <row r="101">
@@ -5291,13 +5291,13 @@
         <v>0</v>
       </c>
       <c r="L101" t="n">
-        <v>506.1099999999994</v>
+        <v>506.11</v>
       </c>
       <c r="M101" t="n">
-        <v>508.6299999999994</v>
+        <v>508.63</v>
       </c>
       <c r="N101" t="n">
-        <v>506.1099999999994</v>
+        <v>506.11</v>
       </c>
     </row>
     <row r="102">
@@ -5333,19 +5333,19 @@
         <v>504.6</v>
       </c>
       <c r="J102" t="n">
-        <v>508.6299999999983</v>
+        <v>508.63</v>
       </c>
       <c r="K102" t="n">
-        <v>4.029999999998267</v>
+        <v>4.029999999999973</v>
       </c>
       <c r="L102" t="n">
-        <v>515.1399999999983</v>
+        <v>515.14</v>
       </c>
       <c r="M102" t="n">
-        <v>517.6599999999983</v>
+        <v>517.66</v>
       </c>
       <c r="N102" t="n">
-        <v>515.1399999999983</v>
+        <v>515.14</v>
       </c>
     </row>
     <row r="103">
@@ -5381,16 +5381,16 @@
         <v>509.6</v>
       </c>
       <c r="J103" t="n">
-        <v>531.3599999999909</v>
+        <v>531.3599999999974</v>
       </c>
       <c r="K103" t="n">
-        <v>21.7599999999909</v>
+        <v>21.75999999999738</v>
       </c>
       <c r="L103" t="n">
-        <v>537.8699999999909</v>
+        <v>537.8699999999974</v>
       </c>
       <c r="M103" t="n">
-        <v>540.3899999999909</v>
+        <v>540.3899999999974</v>
       </c>
       <c r="N103" t="n">
         <v>546.9</v>
@@ -5429,16 +5429,16 @@
         <v>514.6</v>
       </c>
       <c r="J104" t="n">
-        <v>540.3899999999909</v>
+        <v>540.3899999999974</v>
       </c>
       <c r="K104" t="n">
-        <v>25.78999999999087</v>
+        <v>25.78999999999735</v>
       </c>
       <c r="L104" t="n">
         <v>546.9</v>
       </c>
       <c r="M104" t="n">
-        <v>549.4199999999909</v>
+        <v>549.4199999999973</v>
       </c>
       <c r="N104" t="n">
         <v>546.9</v>

</xml_diff>